<commit_message>
📊 BIST Screener | 13.04.2026 16:30 | 606 hisse
</commit_message>
<xml_diff>
--- a/data/bist_screener_2026-04-13.xlsx
+++ b/data/bist_screener_2026-04-13.xlsx
@@ -25699,23 +25699,21 @@
     <row r="581">
       <c r="A581" s="6" t="inlineStr">
         <is>
-          <t>ICUGS</t>
+          <t>BESTE</t>
         </is>
       </c>
       <c r="B581" s="7" t="n">
-        <v>3.91</v>
+        <v>23.4</v>
       </c>
       <c r="C581" s="8" t="n">
-        <v>0.0654</v>
+        <v>-0.0059</v>
       </c>
       <c r="D581" s="9" t="n">
-        <v>69940000</v>
-      </c>
-      <c r="E581" s="8" t="n">
-        <v>0.8667</v>
-      </c>
+        <v>16520000</v>
+      </c>
+      <c r="E581" s="6" t="inlineStr"/>
       <c r="F581" s="7" t="n">
-        <v>68.12</v>
+        <v>53.37</v>
       </c>
       <c r="G581" s="6" t="inlineStr"/>
       <c r="H581" s="6" t="inlineStr"/>
@@ -25723,12 +25721,12 @@
       <c r="J581" s="6" t="inlineStr"/>
       <c r="K581" s="6" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Elektrik, Su, Gaz Hizmetleri</t>
         </is>
       </c>
       <c r="L581" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HOLDING VE YATIRIM, BIST MALİ, BIST ANA</t>
+          <t>BIST ELEKTRIK, BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
         </is>
       </c>
       <c r="M581" s="6" t="inlineStr"/>
@@ -25736,23 +25734,23 @@
     <row r="582">
       <c r="A582" s="2" t="inlineStr">
         <is>
-          <t>INTEK</t>
+          <t>ICUGS</t>
         </is>
       </c>
       <c r="B582" s="3" t="n">
-        <v>254</v>
+        <v>3.91</v>
       </c>
       <c r="C582" s="4" t="n">
-        <v>0.0292</v>
+        <v>0.0654</v>
       </c>
       <c r="D582" s="5" t="n">
-        <v>8560</v>
+        <v>69940000</v>
       </c>
       <c r="E582" s="4" t="n">
-        <v>0.2578</v>
+        <v>0.8667</v>
       </c>
       <c r="F582" s="3" t="n">
-        <v>49.66</v>
+        <v>68.12</v>
       </c>
       <c r="G582" s="2" t="inlineStr"/>
       <c r="H582" s="2" t="inlineStr"/>
@@ -25760,27 +25758,35 @@
       <c r="J582" s="2" t="inlineStr"/>
       <c r="K582" s="2" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
-        </is>
-      </c>
-      <c r="L582" s="2" t="inlineStr"/>
+          <t>Finans</t>
+        </is>
+      </c>
+      <c r="L582" s="2" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST TÜM, BIST HOLDING VE YATIRIM, BIST MALİ, BIST ANA</t>
+        </is>
+      </c>
       <c r="M582" s="2" t="inlineStr"/>
     </row>
     <row r="583">
       <c r="A583" s="6" t="inlineStr">
         <is>
-          <t>ENPRA</t>
+          <t>DMLKT</t>
         </is>
       </c>
       <c r="B583" s="7" t="n">
-        <v>112.4</v>
+        <v>6.28</v>
       </c>
       <c r="C583" s="8" t="n">
-        <v>-0.09939999999999999</v>
-      </c>
-      <c r="D583" s="6" t="inlineStr"/>
+        <v>-0.0048</v>
+      </c>
+      <c r="D583" s="9" t="n">
+        <v>14350000</v>
+      </c>
       <c r="E583" s="6" t="inlineStr"/>
-      <c r="F583" s="6" t="inlineStr"/>
+      <c r="F583" s="7" t="n">
+        <v>83.08</v>
+      </c>
       <c r="G583" s="6" t="inlineStr"/>
       <c r="H583" s="6" t="inlineStr"/>
       <c r="I583" s="6" t="inlineStr"/>
@@ -25796,36 +25802,42 @@
     <row r="584">
       <c r="A584" s="2" t="inlineStr">
         <is>
-          <t>AKGRT</t>
+          <t>BERA</t>
         </is>
       </c>
       <c r="B584" s="3" t="n">
-        <v>7.43</v>
+        <v>17.21</v>
       </c>
       <c r="C584" s="4" t="n">
-        <v>-0.0107</v>
+        <v>-0.0205</v>
       </c>
       <c r="D584" s="5" t="n">
-        <v>12600000</v>
+        <v>12540000</v>
       </c>
       <c r="E584" s="4" t="n">
-        <v>0.28</v>
+        <v>0.9246</v>
       </c>
       <c r="F584" s="3" t="n">
-        <v>48.48</v>
-      </c>
-      <c r="G584" s="2" t="inlineStr"/>
+        <v>46.95</v>
+      </c>
+      <c r="G584" s="3" t="n">
+        <v>162.67</v>
+      </c>
       <c r="H584" s="2" t="inlineStr"/>
-      <c r="I584" s="2" t="inlineStr"/>
-      <c r="J584" s="2" t="inlineStr"/>
+      <c r="I584" s="4" t="n">
+        <v>0.0028</v>
+      </c>
+      <c r="J584" s="4" t="n">
+        <v>-10.3171</v>
+      </c>
       <c r="K584" s="2" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Üretici imalatı</t>
         </is>
       </c>
       <c r="L584" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST SİGORTA, BIST MALİ, BIST YILDIZ, BIST SÜRDÜRÜLEBİLİRLİK</t>
+          <t>BIST TUM-100, BIST TÜM, BIST HOLDING VE YATIRIM, BIST MALİ, BIST KATILIM 100, BIST KATILIM TÜM, BIST YILDIZ, BIST KATILIM 50, BIST KONYA</t>
         </is>
       </c>
       <c r="M584" s="2" t="inlineStr"/>
@@ -25833,104 +25845,102 @@
     <row r="585">
       <c r="A585" s="6" t="inlineStr">
         <is>
-          <t>ALTIN</t>
+          <t>LXGYO</t>
         </is>
       </c>
       <c r="B585" s="7" t="n">
-        <v>80.59999999999999</v>
+        <v>15.85</v>
       </c>
       <c r="C585" s="8" t="n">
-        <v>-0.0154</v>
+        <v>-0.0682</v>
       </c>
       <c r="D585" s="9" t="n">
-        <v>12490000</v>
+        <v>120100000</v>
       </c>
       <c r="E585" s="6" t="inlineStr"/>
       <c r="F585" s="7" t="n">
-        <v>39.07</v>
+        <v>51.61</v>
       </c>
       <c r="G585" s="6" t="inlineStr"/>
       <c r="H585" s="6" t="inlineStr"/>
       <c r="I585" s="6" t="inlineStr"/>
       <c r="J585" s="6" t="inlineStr"/>
-      <c r="K585" s="6" t="inlineStr"/>
-      <c r="L585" s="6" t="inlineStr"/>
+      <c r="K585" s="6" t="inlineStr">
+        <is>
+          <t>Finans</t>
+        </is>
+      </c>
+      <c r="L585" s="6" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST ANA</t>
+        </is>
+      </c>
       <c r="M585" s="6" t="inlineStr"/>
     </row>
     <row r="586">
       <c r="A586" s="2" t="inlineStr">
         <is>
-          <t>BERA</t>
+          <t>ALTIN</t>
         </is>
       </c>
       <c r="B586" s="3" t="n">
-        <v>17.21</v>
+        <v>80.59999999999999</v>
       </c>
       <c r="C586" s="4" t="n">
-        <v>-0.0205</v>
+        <v>-0.0154</v>
       </c>
       <c r="D586" s="5" t="n">
-        <v>12540000</v>
-      </c>
-      <c r="E586" s="4" t="n">
-        <v>0.9246</v>
-      </c>
+        <v>12490000</v>
+      </c>
+      <c r="E586" s="2" t="inlineStr"/>
       <c r="F586" s="3" t="n">
-        <v>46.95</v>
-      </c>
-      <c r="G586" s="3" t="n">
-        <v>162.67</v>
-      </c>
+        <v>39.07</v>
+      </c>
+      <c r="G586" s="2" t="inlineStr"/>
       <c r="H586" s="2" t="inlineStr"/>
-      <c r="I586" s="4" t="n">
-        <v>0.0028</v>
-      </c>
-      <c r="J586" s="4" t="n">
-        <v>-10.3171</v>
-      </c>
-      <c r="K586" s="2" t="inlineStr">
-        <is>
-          <t>Üretici imalatı</t>
-        </is>
-      </c>
-      <c r="L586" s="2" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HOLDING VE YATIRIM, BIST MALİ, BIST KATILIM 100, BIST KATILIM TÜM, BIST YILDIZ, BIST KATILIM 50, BIST KONYA</t>
-        </is>
-      </c>
+      <c r="I586" s="2" t="inlineStr"/>
+      <c r="J586" s="2" t="inlineStr"/>
+      <c r="K586" s="2" t="inlineStr"/>
+      <c r="L586" s="2" t="inlineStr"/>
       <c r="M586" s="2" t="inlineStr"/>
     </row>
     <row r="587">
       <c r="A587" s="6" t="inlineStr">
         <is>
-          <t>SVGYO</t>
+          <t>CRFSA</t>
         </is>
       </c>
       <c r="B587" s="7" t="n">
-        <v>16.35</v>
+        <v>166.6</v>
       </c>
       <c r="C587" s="8" t="n">
-        <v>-0.09970000000000001</v>
+        <v>0.08039999999999999</v>
       </c>
       <c r="D587" s="9" t="n">
-        <v>87640000</v>
-      </c>
-      <c r="E587" s="6" t="inlineStr"/>
+        <v>1310000</v>
+      </c>
+      <c r="E587" s="8" t="n">
+        <v>0.1071</v>
+      </c>
       <c r="F587" s="7" t="n">
-        <v>76.05</v>
+        <v>77.11</v>
       </c>
       <c r="G587" s="6" t="inlineStr"/>
       <c r="H587" s="6" t="inlineStr"/>
-      <c r="I587" s="6" t="inlineStr"/>
-      <c r="J587" s="6" t="inlineStr"/>
+      <c r="I587" s="8" t="n">
+        <v>-3.6635</v>
+      </c>
+      <c r="J587" s="8" t="n">
+        <v>-0.4897</v>
+      </c>
       <c r="K587" s="6" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Perakende satış</t>
         </is>
       </c>
       <c r="L587" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST ANA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST ANA</t>
         </is>
       </c>
       <c r="M587" s="6" t="inlineStr"/>
@@ -25938,21 +25948,21 @@
     <row r="588">
       <c r="A588" s="2" t="inlineStr">
         <is>
-          <t>LXGYO</t>
+          <t>CGCAM</t>
         </is>
       </c>
       <c r="B588" s="3" t="n">
-        <v>15.85</v>
+        <v>36.48</v>
       </c>
       <c r="C588" s="4" t="n">
-        <v>-0.0682</v>
+        <v>-0.0375</v>
       </c>
       <c r="D588" s="5" t="n">
-        <v>120100000</v>
+        <v>6760000</v>
       </c>
       <c r="E588" s="2" t="inlineStr"/>
       <c r="F588" s="3" t="n">
-        <v>51.61</v>
+        <v>50.48</v>
       </c>
       <c r="G588" s="2" t="inlineStr"/>
       <c r="H588" s="2" t="inlineStr"/>
@@ -25960,12 +25970,12 @@
       <c r="J588" s="2" t="inlineStr"/>
       <c r="K588" s="2" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Dayanıklı tüketim malları</t>
         </is>
       </c>
       <c r="L588" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST ANA</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST TAŞ TOPRAK, BIST HALKA ARZ, BIST ANA, BIST MANİSA</t>
         </is>
       </c>
       <c r="M588" s="2" t="inlineStr"/>
@@ -25973,38 +25983,34 @@
     <row r="589">
       <c r="A589" s="6" t="inlineStr">
         <is>
-          <t>EFOR</t>
+          <t>MARMR</t>
         </is>
       </c>
       <c r="B589" s="7" t="n">
-        <v>5.57</v>
+        <v>2.85</v>
       </c>
       <c r="C589" s="8" t="n">
-        <v>0.0431</v>
+        <v>-0.0404</v>
       </c>
       <c r="D589" s="9" t="n">
-        <v>185340000</v>
-      </c>
-      <c r="E589" s="8" t="n">
-        <v>0.2478</v>
-      </c>
+        <v>328740000</v>
+      </c>
+      <c r="E589" s="6" t="inlineStr"/>
       <c r="F589" s="7" t="n">
-        <v>15.58</v>
+        <v>58.27</v>
       </c>
       <c r="G589" s="6" t="inlineStr"/>
       <c r="H589" s="6" t="inlineStr"/>
-      <c r="I589" s="8" t="n">
-        <v>-0.0005999999999999999</v>
-      </c>
+      <c r="I589" s="6" t="inlineStr"/>
       <c r="J589" s="6" t="inlineStr"/>
       <c r="K589" s="6" t="inlineStr">
         <is>
-          <t>Dayanıklı olmayan tüketici ürünleri</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L589" s="6" t="inlineStr">
         <is>
-          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST GIDA ICECEK, BIST SINAI, BIST TÜM, BIST HALKA ARZ, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST ANA, BIST KOCAELI</t>
         </is>
       </c>
       <c r="M589" s="6" t="inlineStr"/>
@@ -26012,21 +26018,21 @@
     <row r="590">
       <c r="A590" s="2" t="inlineStr">
         <is>
-          <t>MARMR</t>
+          <t>SMRVA</t>
         </is>
       </c>
       <c r="B590" s="3" t="n">
-        <v>2.85</v>
+        <v>82.5</v>
       </c>
       <c r="C590" s="4" t="n">
-        <v>-0.0404</v>
+        <v>0.1</v>
       </c>
       <c r="D590" s="5" t="n">
-        <v>328740000</v>
+        <v>6190000</v>
       </c>
       <c r="E590" s="2" t="inlineStr"/>
       <c r="F590" s="3" t="n">
-        <v>58.27</v>
+        <v>73.01000000000001</v>
       </c>
       <c r="G590" s="2" t="inlineStr"/>
       <c r="H590" s="2" t="inlineStr"/>
@@ -26034,12 +26040,12 @@
       <c r="J590" s="2" t="inlineStr"/>
       <c r="K590" s="2" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Ticari hizmetler</t>
         </is>
       </c>
       <c r="L590" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST ANA, BIST KOCAELI</t>
+          <t>BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST MALİ, BIST ANA, BIST TEMETTU</t>
         </is>
       </c>
       <c r="M590" s="2" t="inlineStr"/>
@@ -26047,40 +26053,38 @@
     <row r="591">
       <c r="A591" s="6" t="inlineStr">
         <is>
-          <t>BORLS</t>
+          <t>EFOR</t>
         </is>
       </c>
       <c r="B591" s="7" t="n">
-        <v>4.38</v>
+        <v>5.57</v>
       </c>
       <c r="C591" s="8" t="n">
-        <v>0.0977</v>
+        <v>0.0431</v>
       </c>
       <c r="D591" s="9" t="n">
-        <v>39060000</v>
+        <v>185340000</v>
       </c>
       <c r="E591" s="8" t="n">
-        <v>0.1672</v>
+        <v>0.2478</v>
       </c>
       <c r="F591" s="7" t="n">
-        <v>81.56</v>
+        <v>15.58</v>
       </c>
       <c r="G591" s="6" t="inlineStr"/>
       <c r="H591" s="6" t="inlineStr"/>
       <c r="I591" s="8" t="n">
-        <v>-5.3262</v>
-      </c>
-      <c r="J591" s="8" t="n">
-        <v>-4.2562</v>
-      </c>
+        <v>-0.0005999999999999999</v>
+      </c>
+      <c r="J591" s="6" t="inlineStr"/>
       <c r="K591" s="6" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Dayanıklı olmayan tüketici ürünleri</t>
         </is>
       </c>
       <c r="L591" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HİZMETLER, BIST İSTANBUL, BIST YILDIZ</t>
+          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST GIDA ICECEK, BIST SINAI, BIST TÜM, BIST HALKA ARZ, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50</t>
         </is>
       </c>
       <c r="M591" s="6" t="inlineStr"/>
@@ -26088,34 +26092,40 @@
     <row r="592">
       <c r="A592" s="2" t="inlineStr">
         <is>
-          <t>FRMPL</t>
+          <t>BORLS</t>
         </is>
       </c>
       <c r="B592" s="3" t="n">
-        <v>32.96</v>
+        <v>4.38</v>
       </c>
       <c r="C592" s="4" t="n">
-        <v>-0.009000000000000001</v>
+        <v>0.0977</v>
       </c>
       <c r="D592" s="5" t="n">
-        <v>5490000</v>
-      </c>
-      <c r="E592" s="2" t="inlineStr"/>
+        <v>39060000</v>
+      </c>
+      <c r="E592" s="4" t="n">
+        <v>0.1672</v>
+      </c>
       <c r="F592" s="3" t="n">
-        <v>52.75</v>
+        <v>81.56</v>
       </c>
       <c r="G592" s="2" t="inlineStr"/>
       <c r="H592" s="2" t="inlineStr"/>
-      <c r="I592" s="2" t="inlineStr"/>
-      <c r="J592" s="2" t="inlineStr"/>
+      <c r="I592" s="4" t="n">
+        <v>-5.3262</v>
+      </c>
+      <c r="J592" s="4" t="n">
+        <v>-4.2562</v>
+      </c>
       <c r="K592" s="2" t="inlineStr">
         <is>
-          <t>Üretici imalatı</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L592" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST TEKİRDAĞ</t>
+          <t>BIST TUM-100, BIST TÜM, BIST HİZMETLER, BIST İSTANBUL, BIST YILDIZ</t>
         </is>
       </c>
       <c r="M592" s="2" t="inlineStr"/>
@@ -26123,34 +26133,38 @@
     <row r="593">
       <c r="A593" s="6" t="inlineStr">
         <is>
-          <t>GLRMK</t>
+          <t>NETAS</t>
         </is>
       </c>
       <c r="B593" s="7" t="n">
-        <v>232</v>
+        <v>61</v>
       </c>
       <c r="C593" s="8" t="n">
-        <v>-0.0353</v>
+        <v>-0.0224</v>
       </c>
       <c r="D593" s="9" t="n">
-        <v>14610000</v>
-      </c>
-      <c r="E593" s="6" t="inlineStr"/>
+        <v>1050000</v>
+      </c>
+      <c r="E593" s="8" t="n">
+        <v>0.3695000000000001</v>
+      </c>
       <c r="F593" s="7" t="n">
-        <v>73.84</v>
+        <v>54.08</v>
       </c>
       <c r="G593" s="6" t="inlineStr"/>
       <c r="H593" s="6" t="inlineStr"/>
       <c r="I593" s="6" t="inlineStr"/>
-      <c r="J593" s="6" t="inlineStr"/>
+      <c r="J593" s="8" t="n">
+        <v>0.4139</v>
+      </c>
       <c r="K593" s="6" t="inlineStr">
         <is>
-          <t>Endüstriyel hizmetler</t>
+          <t>Teknoloji hizmetleri</t>
         </is>
       </c>
       <c r="L593" s="6" t="inlineStr">
         <is>
-          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50, BIST KATILIM 30, BIST ANKARA, BIST KATILIM 30 EŞİT AĞIRLIKLI GETİRİ</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST İSTANBUL, BIST KATILIM 100, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KURUMSAL YÖNETİM</t>
         </is>
       </c>
       <c r="M593" s="6" t="inlineStr"/>
@@ -26158,21 +26172,21 @@
     <row r="594">
       <c r="A594" s="2" t="inlineStr">
         <is>
-          <t>MCARD</t>
+          <t>FRMPL</t>
         </is>
       </c>
       <c r="B594" s="3" t="n">
-        <v>197</v>
+        <v>32.96</v>
       </c>
       <c r="C594" s="4" t="n">
-        <v>0.0336</v>
+        <v>-0.009000000000000001</v>
       </c>
       <c r="D594" s="5" t="n">
-        <v>14110000</v>
+        <v>5490000</v>
       </c>
       <c r="E594" s="2" t="inlineStr"/>
       <c r="F594" s="3" t="n">
-        <v>77.95999999999999</v>
+        <v>52.75</v>
       </c>
       <c r="G594" s="2" t="inlineStr"/>
       <c r="H594" s="2" t="inlineStr"/>
@@ -26180,12 +26194,12 @@
       <c r="J594" s="2" t="inlineStr"/>
       <c r="K594" s="2" t="inlineStr">
         <is>
-          <t>Ticari hizmetler</t>
+          <t>Üretici imalatı</t>
         </is>
       </c>
       <c r="L594" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST TEKİRDAĞ</t>
         </is>
       </c>
       <c r="M594" s="2" t="inlineStr"/>
@@ -26193,38 +26207,34 @@
     <row r="595">
       <c r="A595" s="6" t="inlineStr">
         <is>
-          <t>NETAS</t>
+          <t>SVGYO</t>
         </is>
       </c>
       <c r="B595" s="7" t="n">
-        <v>61</v>
+        <v>16.35</v>
       </c>
       <c r="C595" s="8" t="n">
-        <v>-0.0224</v>
+        <v>-0.09970000000000001</v>
       </c>
       <c r="D595" s="9" t="n">
-        <v>1050000</v>
-      </c>
-      <c r="E595" s="8" t="n">
-        <v>0.3695000000000001</v>
-      </c>
+        <v>87640000</v>
+      </c>
+      <c r="E595" s="6" t="inlineStr"/>
       <c r="F595" s="7" t="n">
-        <v>54.08</v>
+        <v>76.05</v>
       </c>
       <c r="G595" s="6" t="inlineStr"/>
       <c r="H595" s="6" t="inlineStr"/>
       <c r="I595" s="6" t="inlineStr"/>
-      <c r="J595" s="8" t="n">
-        <v>0.4139</v>
-      </c>
+      <c r="J595" s="6" t="inlineStr"/>
       <c r="K595" s="6" t="inlineStr">
         <is>
-          <t>Teknoloji hizmetleri</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L595" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST İSTANBUL, BIST KATILIM 100, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KURUMSAL YÖNETİM</t>
+          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST ANA</t>
         </is>
       </c>
       <c r="M595" s="6" t="inlineStr"/>
@@ -26232,69 +26242,77 @@
     <row r="596">
       <c r="A596" s="2" t="inlineStr">
         <is>
-          <t>BESTE</t>
+          <t>MMCAS</t>
         </is>
       </c>
       <c r="B596" s="3" t="n">
-        <v>23.4</v>
+        <v>79.90000000000001</v>
       </c>
       <c r="C596" s="4" t="n">
-        <v>-0.0059</v>
+        <v>0.0296</v>
       </c>
       <c r="D596" s="5" t="n">
-        <v>16520000</v>
-      </c>
-      <c r="E596" s="2" t="inlineStr"/>
+        <v>32000</v>
+      </c>
+      <c r="E596" s="4" t="n">
+        <v>0.58</v>
+      </c>
       <c r="F596" s="3" t="n">
-        <v>53.37</v>
+        <v>36.74</v>
       </c>
       <c r="G596" s="2" t="inlineStr"/>
       <c r="H596" s="2" t="inlineStr"/>
-      <c r="I596" s="2" t="inlineStr"/>
-      <c r="J596" s="2" t="inlineStr"/>
+      <c r="I596" s="4" t="n">
+        <v>-9.409700000000001</v>
+      </c>
+      <c r="J596" s="4" t="n">
+        <v>-4.155</v>
+      </c>
       <c r="K596" s="2" t="inlineStr">
         <is>
-          <t>Elektrik, Su, Gaz Hizmetleri</t>
-        </is>
-      </c>
-      <c r="L596" s="2" t="inlineStr">
-        <is>
-          <t>BIST ELEKTRIK, BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
-        </is>
-      </c>
+          <t>Taşımacılık</t>
+        </is>
+      </c>
+      <c r="L596" s="2" t="inlineStr"/>
       <c r="M596" s="2" t="inlineStr"/>
     </row>
     <row r="597">
       <c r="A597" s="6" t="inlineStr">
         <is>
-          <t>SMRVA</t>
+          <t>ARZUM</t>
         </is>
       </c>
       <c r="B597" s="7" t="n">
-        <v>82.5</v>
+        <v>3.27</v>
       </c>
       <c r="C597" s="8" t="n">
-        <v>0.1</v>
+        <v>-0.0325</v>
       </c>
       <c r="D597" s="9" t="n">
-        <v>6190000</v>
-      </c>
-      <c r="E597" s="6" t="inlineStr"/>
+        <v>73930000</v>
+      </c>
+      <c r="E597" s="8" t="n">
+        <v>0.7119</v>
+      </c>
       <c r="F597" s="7" t="n">
-        <v>73.01000000000001</v>
+        <v>62.53</v>
       </c>
       <c r="G597" s="6" t="inlineStr"/>
       <c r="H597" s="6" t="inlineStr"/>
-      <c r="I597" s="6" t="inlineStr"/>
-      <c r="J597" s="6" t="inlineStr"/>
+      <c r="I597" s="8" t="n">
+        <v>-191.6342</v>
+      </c>
+      <c r="J597" s="8" t="n">
+        <v>-0.8093</v>
+      </c>
       <c r="K597" s="6" t="inlineStr">
         <is>
-          <t>Ticari hizmetler</t>
+          <t>Dağıtım servisleri</t>
         </is>
       </c>
       <c r="L597" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST MALİ, BIST ANA, BIST TEMETTU</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST İSTANBUL, BIST ANA, BIST KURUMSAL YÖNETİM</t>
         </is>
       </c>
       <c r="M597" s="6" t="inlineStr"/>
@@ -26333,21 +26351,21 @@
     <row r="599">
       <c r="A599" s="6" t="inlineStr">
         <is>
-          <t>GENKM</t>
+          <t>EMPAE</t>
         </is>
       </c>
       <c r="B599" s="7" t="n">
-        <v>13.48</v>
+        <v>40.02</v>
       </c>
       <c r="C599" s="8" t="n">
-        <v>-0.0288</v>
+        <v>-0.0471</v>
       </c>
       <c r="D599" s="9" t="n">
-        <v>60540000</v>
+        <v>17300000</v>
       </c>
       <c r="E599" s="6" t="inlineStr"/>
       <c r="F599" s="7" t="n">
-        <v>52.54</v>
+        <v>53.04</v>
       </c>
       <c r="G599" s="6" t="inlineStr"/>
       <c r="H599" s="6" t="inlineStr"/>
@@ -26355,12 +26373,12 @@
       <c r="J599" s="6" t="inlineStr"/>
       <c r="K599" s="6" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
+          <t>Elektronik teknoloji</t>
         </is>
       </c>
       <c r="L599" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST KOCAELI</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI</t>
         </is>
       </c>
       <c r="M599" s="6" t="inlineStr"/>
@@ -26368,64 +26386,48 @@
     <row r="600">
       <c r="A600" s="2" t="inlineStr">
         <is>
-          <t>CRFSA</t>
+          <t>ENPRA</t>
         </is>
       </c>
       <c r="B600" s="3" t="n">
-        <v>166.6</v>
+        <v>112.4</v>
       </c>
       <c r="C600" s="4" t="n">
-        <v>0.08039999999999999</v>
-      </c>
-      <c r="D600" s="5" t="n">
-        <v>1310000</v>
-      </c>
-      <c r="E600" s="4" t="n">
-        <v>0.1071</v>
-      </c>
-      <c r="F600" s="3" t="n">
-        <v>77.11</v>
-      </c>
+        <v>-0.09939999999999999</v>
+      </c>
+      <c r="D600" s="2" t="inlineStr"/>
+      <c r="E600" s="2" t="inlineStr"/>
+      <c r="F600" s="2" t="inlineStr"/>
       <c r="G600" s="2" t="inlineStr"/>
       <c r="H600" s="2" t="inlineStr"/>
-      <c r="I600" s="4" t="n">
-        <v>-3.6635</v>
-      </c>
-      <c r="J600" s="4" t="n">
-        <v>-0.4897</v>
-      </c>
+      <c r="I600" s="2" t="inlineStr"/>
+      <c r="J600" s="2" t="inlineStr"/>
       <c r="K600" s="2" t="inlineStr">
         <is>
-          <t>Perakende satış</t>
-        </is>
-      </c>
-      <c r="L600" s="2" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST ANA</t>
-        </is>
-      </c>
+          <t>Finans</t>
+        </is>
+      </c>
+      <c r="L600" s="2" t="inlineStr"/>
       <c r="M600" s="2" t="inlineStr"/>
     </row>
     <row r="601">
       <c r="A601" s="6" t="inlineStr">
         <is>
-          <t>UCAYM</t>
+          <t>MCARD</t>
         </is>
       </c>
       <c r="B601" s="7" t="n">
-        <v>29.72</v>
+        <v>197</v>
       </c>
       <c r="C601" s="8" t="n">
-        <v>0.0599</v>
+        <v>0.0336</v>
       </c>
       <c r="D601" s="9" t="n">
-        <v>11110000</v>
-      </c>
-      <c r="E601" s="8" t="n">
-        <v>0.2667</v>
-      </c>
+        <v>14110000</v>
+      </c>
+      <c r="E601" s="6" t="inlineStr"/>
       <c r="F601" s="7" t="n">
-        <v>61.87</v>
+        <v>77.95999999999999</v>
       </c>
       <c r="G601" s="6" t="inlineStr"/>
       <c r="H601" s="6" t="inlineStr"/>
@@ -26433,12 +26435,12 @@
       <c r="J601" s="6" t="inlineStr"/>
       <c r="K601" s="6" t="inlineStr">
         <is>
-          <t>Endüstriyel hizmetler</t>
+          <t>Ticari hizmetler</t>
         </is>
       </c>
       <c r="L601" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI</t>
         </is>
       </c>
       <c r="M601" s="6" t="inlineStr"/>
@@ -26446,40 +26448,36 @@
     <row r="602">
       <c r="A602" s="2" t="inlineStr">
         <is>
-          <t>ARZUM</t>
+          <t>UCAYM</t>
         </is>
       </c>
       <c r="B602" s="3" t="n">
-        <v>3.27</v>
+        <v>29.72</v>
       </c>
       <c r="C602" s="4" t="n">
-        <v>-0.0325</v>
+        <v>0.0599</v>
       </c>
       <c r="D602" s="5" t="n">
-        <v>73930000</v>
+        <v>11110000</v>
       </c>
       <c r="E602" s="4" t="n">
-        <v>0.7119</v>
+        <v>0.2667</v>
       </c>
       <c r="F602" s="3" t="n">
-        <v>62.53</v>
+        <v>61.87</v>
       </c>
       <c r="G602" s="2" t="inlineStr"/>
       <c r="H602" s="2" t="inlineStr"/>
-      <c r="I602" s="4" t="n">
-        <v>-191.6342</v>
-      </c>
-      <c r="J602" s="4" t="n">
-        <v>-0.8093</v>
-      </c>
+      <c r="I602" s="2" t="inlineStr"/>
+      <c r="J602" s="2" t="inlineStr"/>
       <c r="K602" s="2" t="inlineStr">
         <is>
-          <t>Dağıtım servisleri</t>
+          <t>Endüstriyel hizmetler</t>
         </is>
       </c>
       <c r="L602" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST İSTANBUL, BIST ANA, BIST KURUMSAL YÖNETİM</t>
+          <t>BIST TUM-100, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
         </is>
       </c>
       <c r="M602" s="2" t="inlineStr"/>
@@ -26487,29 +26485,35 @@
     <row r="603">
       <c r="A603" s="6" t="inlineStr">
         <is>
-          <t>DMLKT</t>
+          <t>BRMEN</t>
         </is>
       </c>
       <c r="B603" s="7" t="n">
-        <v>6.28</v>
+        <v>10</v>
       </c>
       <c r="C603" s="8" t="n">
-        <v>-0.0048</v>
+        <v>-0.0476</v>
       </c>
       <c r="D603" s="9" t="n">
-        <v>14350000</v>
-      </c>
-      <c r="E603" s="6" t="inlineStr"/>
+        <v>266560</v>
+      </c>
+      <c r="E603" s="8" t="n">
+        <v>0.95</v>
+      </c>
       <c r="F603" s="7" t="n">
-        <v>83.08</v>
+        <v>59.22</v>
       </c>
       <c r="G603" s="6" t="inlineStr"/>
       <c r="H603" s="6" t="inlineStr"/>
-      <c r="I603" s="6" t="inlineStr"/>
-      <c r="J603" s="6" t="inlineStr"/>
+      <c r="I603" s="8" t="n">
+        <v>-23.6291</v>
+      </c>
+      <c r="J603" s="8" t="n">
+        <v>-0.4678</v>
+      </c>
       <c r="K603" s="6" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>İşlenebilen endüstriler</t>
         </is>
       </c>
       <c r="L603" s="6" t="inlineStr"/>
@@ -26518,58 +26522,58 @@
     <row r="604">
       <c r="A604" s="2" t="inlineStr">
         <is>
-          <t>MMCAS</t>
+          <t>GLRMK</t>
         </is>
       </c>
       <c r="B604" s="3" t="n">
-        <v>79.90000000000001</v>
+        <v>232</v>
       </c>
       <c r="C604" s="4" t="n">
-        <v>0.0296</v>
+        <v>-0.0353</v>
       </c>
       <c r="D604" s="5" t="n">
-        <v>32000</v>
-      </c>
-      <c r="E604" s="4" t="n">
-        <v>0.58</v>
-      </c>
+        <v>14610000</v>
+      </c>
+      <c r="E604" s="2" t="inlineStr"/>
       <c r="F604" s="3" t="n">
-        <v>36.74</v>
+        <v>73.84</v>
       </c>
       <c r="G604" s="2" t="inlineStr"/>
       <c r="H604" s="2" t="inlineStr"/>
-      <c r="I604" s="4" t="n">
-        <v>-9.409700000000001</v>
-      </c>
-      <c r="J604" s="4" t="n">
-        <v>-4.155</v>
-      </c>
+      <c r="I604" s="2" t="inlineStr"/>
+      <c r="J604" s="2" t="inlineStr"/>
       <c r="K604" s="2" t="inlineStr">
         <is>
-          <t>Taşımacılık</t>
-        </is>
-      </c>
-      <c r="L604" s="2" t="inlineStr"/>
+          <t>Endüstriyel hizmetler</t>
+        </is>
+      </c>
+      <c r="L604" s="2" t="inlineStr">
+        <is>
+          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50, BIST KATILIM 30, BIST ANKARA, BIST KATILIM 30 EŞİT AĞIRLIKLI GETİRİ</t>
+        </is>
+      </c>
       <c r="M604" s="2" t="inlineStr"/>
     </row>
     <row r="605">
       <c r="A605" s="6" t="inlineStr">
         <is>
-          <t>EMPAE</t>
+          <t>INTEK</t>
         </is>
       </c>
       <c r="B605" s="7" t="n">
-        <v>40.02</v>
+        <v>254</v>
       </c>
       <c r="C605" s="8" t="n">
-        <v>-0.0471</v>
+        <v>0.0292</v>
       </c>
       <c r="D605" s="9" t="n">
-        <v>17300000</v>
-      </c>
-      <c r="E605" s="6" t="inlineStr"/>
+        <v>8560</v>
+      </c>
+      <c r="E605" s="8" t="n">
+        <v>0.2578</v>
+      </c>
       <c r="F605" s="7" t="n">
-        <v>53.04</v>
+        <v>49.66</v>
       </c>
       <c r="G605" s="6" t="inlineStr"/>
       <c r="H605" s="6" t="inlineStr"/>
@@ -26577,71 +26581,67 @@
       <c r="J605" s="6" t="inlineStr"/>
       <c r="K605" s="6" t="inlineStr">
         <is>
-          <t>Elektronik teknoloji</t>
-        </is>
-      </c>
-      <c r="L605" s="6" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI</t>
-        </is>
-      </c>
+          <t>İşlenebilen endüstriler</t>
+        </is>
+      </c>
+      <c r="L605" s="6" t="inlineStr"/>
       <c r="M605" s="6" t="inlineStr"/>
     </row>
     <row r="606">
       <c r="A606" s="2" t="inlineStr">
         <is>
-          <t>BRMEN</t>
+          <t>AKGRT</t>
         </is>
       </c>
       <c r="B606" s="3" t="n">
-        <v>10</v>
+        <v>7.43</v>
       </c>
       <c r="C606" s="4" t="n">
-        <v>-0.0476</v>
+        <v>-0.0107</v>
       </c>
       <c r="D606" s="5" t="n">
-        <v>266560</v>
+        <v>12600000</v>
       </c>
       <c r="E606" s="4" t="n">
-        <v>0.95</v>
+        <v>0.28</v>
       </c>
       <c r="F606" s="3" t="n">
-        <v>59.22</v>
+        <v>48.48</v>
       </c>
       <c r="G606" s="2" t="inlineStr"/>
       <c r="H606" s="2" t="inlineStr"/>
-      <c r="I606" s="4" t="n">
-        <v>-23.6291</v>
-      </c>
-      <c r="J606" s="4" t="n">
-        <v>-0.4678</v>
-      </c>
+      <c r="I606" s="2" t="inlineStr"/>
+      <c r="J606" s="2" t="inlineStr"/>
       <c r="K606" s="2" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
-        </is>
-      </c>
-      <c r="L606" s="2" t="inlineStr"/>
+          <t>Finans</t>
+        </is>
+      </c>
+      <c r="L606" s="2" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST TÜM, BIST SİGORTA, BIST MALİ, BIST YILDIZ, BIST SÜRDÜRÜLEBİLİRLİK</t>
+        </is>
+      </c>
       <c r="M606" s="2" t="inlineStr"/>
     </row>
     <row r="607">
       <c r="A607" s="6" t="inlineStr">
         <is>
-          <t>CGCAM</t>
+          <t>GENKM</t>
         </is>
       </c>
       <c r="B607" s="7" t="n">
-        <v>36.48</v>
+        <v>13.48</v>
       </c>
       <c r="C607" s="8" t="n">
-        <v>-0.0375</v>
+        <v>-0.0288</v>
       </c>
       <c r="D607" s="9" t="n">
-        <v>6760000</v>
+        <v>60540000</v>
       </c>
       <c r="E607" s="6" t="inlineStr"/>
       <c r="F607" s="7" t="n">
-        <v>50.48</v>
+        <v>52.54</v>
       </c>
       <c r="G607" s="6" t="inlineStr"/>
       <c r="H607" s="6" t="inlineStr"/>
@@ -26649,12 +26649,12 @@
       <c r="J607" s="6" t="inlineStr"/>
       <c r="K607" s="6" t="inlineStr">
         <is>
-          <t>Dayanıklı tüketim malları</t>
+          <t>İşlenebilen endüstriler</t>
         </is>
       </c>
       <c r="L607" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST TAŞ TOPRAK, BIST HALKA ARZ, BIST ANA, BIST MANİSA</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST KOCAELI</t>
         </is>
       </c>
       <c r="M607" s="6" t="inlineStr"/>
@@ -26681,7 +26681,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>13.04.2026 15:30</t>
+          <t>13.04.2026 16:30</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 BIST Screener | 13.04.2026 19:52 | 606 hisse
</commit_message>
<xml_diff>
--- a/data/bist_screener_2026-04-13.xlsx
+++ b/data/bist_screener_2026-04-13.xlsx
@@ -15123,42 +15123,40 @@
     <row r="337">
       <c r="A337" s="6" t="inlineStr">
         <is>
-          <t>HEKTS</t>
+          <t>BJKAS</t>
         </is>
       </c>
       <c r="B337" s="7" t="n">
-        <v>3.09</v>
+        <v>1.48</v>
       </c>
       <c r="C337" s="8" t="n">
-        <v>0.0131</v>
+        <v>-0.0199</v>
       </c>
       <c r="D337" s="9" t="n">
-        <v>117630000</v>
+        <v>31640000</v>
       </c>
       <c r="E337" s="8" t="n">
-        <v>0.4463</v>
+        <v>0.2988</v>
       </c>
       <c r="F337" s="7" t="n">
-        <v>57.11</v>
+        <v>47.33</v>
       </c>
       <c r="G337" s="6" t="inlineStr"/>
       <c r="H337" s="7" t="n">
-        <v>1.87</v>
+        <v>1.86</v>
       </c>
       <c r="I337" s="8" t="n">
-        <v>-0.2826</v>
-      </c>
-      <c r="J337" s="8" t="n">
-        <v>-0.3658</v>
-      </c>
+        <v>-4.0666</v>
+      </c>
+      <c r="J337" s="6" t="inlineStr"/>
       <c r="K337" s="6" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
+          <t>Tüketici hizmetleri</t>
         </is>
       </c>
       <c r="L337" s="6" t="inlineStr">
         <is>
-          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST SINAI, BIST TÜM, BIST 50, BIST KİMYA PETROL PLASTİK, BIST 100-30, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST SÜRDÜRÜLEBİLİRLİK, BIST 50-30, BIST KOCAELI, BIST 50-30 AGIRLIK SINIRLAMALI 25, BIST 50-30 AĞIRLIK SINIRLAMALI 10</t>
+          <t>BIST TUM-100, BIST TÜM, BIST SPOR, BIST HİZMETLER, BIST İSTANBUL, BIST YILDIZ</t>
         </is>
       </c>
       <c r="M337" s="6" t="inlineStr"/>
@@ -15166,42 +15164,42 @@
     <row r="338">
       <c r="A338" s="2" t="inlineStr">
         <is>
-          <t>KOTON</t>
+          <t>HEKTS</t>
         </is>
       </c>
       <c r="B338" s="3" t="n">
-        <v>15.15</v>
+        <v>3.09</v>
       </c>
       <c r="C338" s="4" t="n">
-        <v>-0.0124</v>
+        <v>0.0131</v>
       </c>
       <c r="D338" s="5" t="n">
-        <v>3570000</v>
+        <v>117630000</v>
       </c>
       <c r="E338" s="4" t="n">
-        <v>0.1318</v>
+        <v>0.4463</v>
       </c>
       <c r="F338" s="3" t="n">
-        <v>51.7</v>
+        <v>57.11</v>
       </c>
       <c r="G338" s="2" t="inlineStr"/>
       <c r="H338" s="3" t="n">
-        <v>1.88</v>
+        <v>1.87</v>
       </c>
       <c r="I338" s="4" t="n">
-        <v>-0.1453</v>
+        <v>-0.2826</v>
       </c>
       <c r="J338" s="4" t="n">
-        <v>-313.1914</v>
+        <v>-0.3658</v>
       </c>
       <c r="K338" s="2" t="inlineStr">
         <is>
-          <t>Dayanıklı olmayan tüketici ürünleri</t>
+          <t>İşlenebilen endüstriler</t>
         </is>
       </c>
       <c r="L338" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST TİCARET, BIST HİZMETLER, BIST KATILIM 100, BIST KATILIM TÜM, BIST YILDIZ</t>
+          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST SINAI, BIST TÜM, BIST 50, BIST KİMYA PETROL PLASTİK, BIST 100-30, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST SÜRDÜRÜLEBİLİRLİK, BIST 50-30, BIST KOCAELI, BIST 50-30 AGIRLIK SINIRLAMALI 25, BIST 50-30 AĞIRLIK SINIRLAMALI 10</t>
         </is>
       </c>
       <c r="M338" s="2" t="inlineStr"/>
@@ -15209,44 +15207,42 @@
     <row r="339">
       <c r="A339" s="6" t="inlineStr">
         <is>
-          <t>YGGYO</t>
+          <t>KOTON</t>
         </is>
       </c>
       <c r="B339" s="7" t="n">
-        <v>209.5</v>
+        <v>15.15</v>
       </c>
       <c r="C339" s="8" t="n">
-        <v>0.0062</v>
+        <v>-0.0124</v>
       </c>
       <c r="D339" s="9" t="n">
-        <v>574930</v>
+        <v>3570000</v>
       </c>
       <c r="E339" s="8" t="n">
-        <v>0.8517</v>
+        <v>0.1318</v>
       </c>
       <c r="F339" s="7" t="n">
-        <v>58.48</v>
-      </c>
-      <c r="G339" s="7" t="n">
-        <v>9.210000000000001</v>
-      </c>
+        <v>51.7</v>
+      </c>
+      <c r="G339" s="6" t="inlineStr"/>
       <c r="H339" s="7" t="n">
-        <v>1.9</v>
+        <v>1.88</v>
       </c>
       <c r="I339" s="8" t="n">
-        <v>0.2608</v>
+        <v>-0.1453</v>
       </c>
       <c r="J339" s="8" t="n">
-        <v>6.3451</v>
+        <v>-313.1914</v>
       </c>
       <c r="K339" s="6" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Dayanıklı olmayan tüketici ürünleri</t>
         </is>
       </c>
       <c r="L339" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST MALİ, BIST YILDIZ</t>
+          <t>BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST TİCARET, BIST HİZMETLER, BIST KATILIM 100, BIST KATILIM TÜM, BIST YILDIZ</t>
         </is>
       </c>
       <c r="M339" s="6" t="inlineStr"/>
@@ -15254,44 +15250,44 @@
     <row r="340">
       <c r="A340" s="2" t="inlineStr">
         <is>
-          <t>EGPRO</t>
+          <t>YGGYO</t>
         </is>
       </c>
       <c r="B340" s="3" t="n">
-        <v>31.2</v>
+        <v>209.5</v>
       </c>
       <c r="C340" s="4" t="n">
-        <v>-0.0064</v>
+        <v>0.0062</v>
       </c>
       <c r="D340" s="5" t="n">
-        <v>1470000</v>
+        <v>574930</v>
       </c>
       <c r="E340" s="4" t="n">
-        <v>0.1314</v>
+        <v>0.8517</v>
       </c>
       <c r="F340" s="3" t="n">
-        <v>62.71</v>
+        <v>58.48</v>
       </c>
       <c r="G340" s="3" t="n">
-        <v>17.01</v>
+        <v>9.210000000000001</v>
       </c>
       <c r="H340" s="3" t="n">
-        <v>1.91</v>
+        <v>1.9</v>
       </c>
       <c r="I340" s="4" t="n">
-        <v>0.132</v>
+        <v>0.2608</v>
       </c>
       <c r="J340" s="4" t="n">
-        <v>0.0143</v>
+        <v>6.3451</v>
       </c>
       <c r="K340" s="2" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L340" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST KATILIM TÜM, BIST YILDIZ, BIST TEMETTU, BIST KATILIM TEMETTU, BIST İZMİR</t>
+          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST MALİ, BIST YILDIZ</t>
         </is>
       </c>
       <c r="M340" s="2" t="inlineStr"/>
@@ -15299,42 +15295,44 @@
     <row r="341">
       <c r="A341" s="6" t="inlineStr">
         <is>
-          <t>KLYPV</t>
+          <t>EGPRO</t>
         </is>
       </c>
       <c r="B341" s="7" t="n">
-        <v>62</v>
+        <v>31.2</v>
       </c>
       <c r="C341" s="8" t="n">
-        <v>-0.0135</v>
+        <v>-0.0064</v>
       </c>
       <c r="D341" s="9" t="n">
-        <v>3670000</v>
+        <v>1470000</v>
       </c>
       <c r="E341" s="8" t="n">
-        <v>0.1126</v>
+        <v>0.1314</v>
       </c>
       <c r="F341" s="7" t="n">
-        <v>57.91</v>
-      </c>
-      <c r="G341" s="6" t="inlineStr"/>
+        <v>62.71</v>
+      </c>
+      <c r="G341" s="7" t="n">
+        <v>17.01</v>
+      </c>
       <c r="H341" s="7" t="n">
-        <v>1.92</v>
+        <v>1.91</v>
       </c>
       <c r="I341" s="8" t="n">
-        <v>-0.06150000000000001</v>
+        <v>0.132</v>
       </c>
       <c r="J341" s="8" t="n">
-        <v>-1.6584</v>
+        <v>0.0143</v>
       </c>
       <c r="K341" s="6" t="inlineStr">
         <is>
-          <t>Üretici imalatı</t>
+          <t>İşlenebilen endüstriler</t>
         </is>
       </c>
       <c r="L341" s="6" t="inlineStr">
         <is>
-          <t>BIST ELEKTRIK, BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST HİZMETLER, BIST YILDIZ, BIST ANKARA</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST KATILIM TÜM, BIST YILDIZ, BIST TEMETTU, BIST KATILIM TEMETTU, BIST İZMİR</t>
         </is>
       </c>
       <c r="M341" s="6" t="inlineStr"/>
@@ -15342,44 +15340,42 @@
     <row r="342">
       <c r="A342" s="2" t="inlineStr">
         <is>
-          <t>OYAKC</t>
+          <t>KLYPV</t>
         </is>
       </c>
       <c r="B342" s="3" t="n">
-        <v>25.16</v>
+        <v>62</v>
       </c>
       <c r="C342" s="4" t="n">
-        <v>-0.0172</v>
+        <v>-0.0135</v>
       </c>
       <c r="D342" s="5" t="n">
-        <v>15100000</v>
+        <v>3670000</v>
       </c>
       <c r="E342" s="4" t="n">
-        <v>0.1995</v>
+        <v>0.1126</v>
       </c>
       <c r="F342" s="3" t="n">
-        <v>58.44</v>
-      </c>
-      <c r="G342" s="3" t="n">
-        <v>14.49</v>
-      </c>
+        <v>57.91</v>
+      </c>
+      <c r="G342" s="2" t="inlineStr"/>
       <c r="H342" s="3" t="n">
-        <v>1.94</v>
+        <v>1.92</v>
       </c>
       <c r="I342" s="4" t="n">
-        <v>0.1553</v>
+        <v>-0.06150000000000001</v>
       </c>
       <c r="J342" s="4" t="n">
-        <v>-0.5638000000000001</v>
+        <v>-1.6584</v>
       </c>
       <c r="K342" s="2" t="inlineStr">
         <is>
-          <t>Enerji-dışı mineraller</t>
+          <t>Üretici imalatı</t>
         </is>
       </c>
       <c r="L342" s="2" t="inlineStr">
         <is>
-          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST SINAI, BIST TÜM, BIST 50, BIST TAŞ TOPRAK, BIST 100-30, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST SÜRDÜRÜLEBİLİRLİK, BIST KURUMSAL YÖNETİM, BIST 50-30, BIST ANKARA, BIST SÜRDÜRÜLEBİLİRLİK 25, BIST 50-30 AGIRLIK SINIRLAMALI 25, BIST 50-30 AĞIRLIK SINIRLAMALI 10</t>
+          <t>BIST ELEKTRIK, BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST HİZMETLER, BIST YILDIZ, BIST ANKARA</t>
         </is>
       </c>
       <c r="M342" s="2" t="inlineStr"/>
@@ -15387,42 +15383,44 @@
     <row r="343">
       <c r="A343" s="6" t="inlineStr">
         <is>
-          <t>KARTN</t>
+          <t>OYAKC</t>
         </is>
       </c>
       <c r="B343" s="7" t="n">
-        <v>64.5</v>
+        <v>25.16</v>
       </c>
       <c r="C343" s="8" t="n">
-        <v>-0.0293</v>
+        <v>-0.0172</v>
       </c>
       <c r="D343" s="9" t="n">
-        <v>617410</v>
+        <v>15100000</v>
       </c>
       <c r="E343" s="8" t="n">
-        <v>0.2187</v>
+        <v>0.1995</v>
       </c>
       <c r="F343" s="7" t="n">
-        <v>41.05</v>
-      </c>
-      <c r="G343" s="6" t="inlineStr"/>
+        <v>58.44</v>
+      </c>
+      <c r="G343" s="7" t="n">
+        <v>14.49</v>
+      </c>
       <c r="H343" s="7" t="n">
-        <v>1.96</v>
+        <v>1.94</v>
       </c>
       <c r="I343" s="8" t="n">
-        <v>-0.4183</v>
+        <v>0.1553</v>
       </c>
       <c r="J343" s="8" t="n">
-        <v>-1.6177</v>
+        <v>-0.5638000000000001</v>
       </c>
       <c r="K343" s="6" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
+          <t>Enerji-dışı mineraller</t>
         </is>
       </c>
       <c r="L343" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST ORMAN KAĞIT BASIM, BIST ANA, BIST KOCAELI</t>
+          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST SINAI, BIST TÜM, BIST 50, BIST TAŞ TOPRAK, BIST 100-30, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST SÜRDÜRÜLEBİLİRLİK, BIST KURUMSAL YÖNETİM, BIST 50-30, BIST ANKARA, BIST SÜRDÜRÜLEBİLİRLİK 25, BIST 50-30 AGIRLIK SINIRLAMALI 25, BIST 50-30 AĞIRLIK SINIRLAMALI 10</t>
         </is>
       </c>
       <c r="M343" s="6" t="inlineStr"/>
@@ -15430,44 +15428,42 @@
     <row r="344">
       <c r="A344" s="2" t="inlineStr">
         <is>
-          <t>TBORG</t>
+          <t>KARTN</t>
         </is>
       </c>
       <c r="B344" s="3" t="n">
-        <v>143.3</v>
+        <v>64.5</v>
       </c>
       <c r="C344" s="4" t="n">
-        <v>-0.0311</v>
+        <v>-0.0293</v>
       </c>
       <c r="D344" s="5" t="n">
-        <v>188410</v>
+        <v>617410</v>
       </c>
       <c r="E344" s="4" t="n">
-        <v>0.0501</v>
+        <v>0.2187</v>
       </c>
       <c r="F344" s="3" t="n">
-        <v>38.54</v>
-      </c>
-      <c r="G344" s="3" t="n">
-        <v>14.31</v>
-      </c>
+        <v>41.05</v>
+      </c>
+      <c r="G344" s="2" t="inlineStr"/>
       <c r="H344" s="3" t="n">
         <v>1.96</v>
       </c>
       <c r="I344" s="4" t="n">
-        <v>0.157</v>
+        <v>-0.4183</v>
       </c>
       <c r="J344" s="4" t="n">
-        <v>-1.2844</v>
+        <v>-1.6177</v>
       </c>
       <c r="K344" s="2" t="inlineStr">
         <is>
-          <t>Dayanıklı olmayan tüketici ürünleri</t>
+          <t>İşlenebilen endüstriler</t>
         </is>
       </c>
       <c r="L344" s="2" t="inlineStr">
         <is>
-          <t>BIST GIDA ICECEK, BIST TUM-100, BIST SINAI, BIST TÜM, BIST ANA, BIST İZMİR</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST ORMAN KAĞIT BASIM, BIST ANA, BIST KOCAELI</t>
         </is>
       </c>
       <c r="M344" s="2" t="inlineStr"/>
@@ -15475,42 +15471,44 @@
     <row r="345">
       <c r="A345" s="6" t="inlineStr">
         <is>
-          <t>EKOS</t>
+          <t>TBORG</t>
         </is>
       </c>
       <c r="B345" s="7" t="n">
-        <v>5.5</v>
+        <v>143.3</v>
       </c>
       <c r="C345" s="8" t="n">
-        <v>-0.0248</v>
+        <v>-0.0311</v>
       </c>
       <c r="D345" s="9" t="n">
-        <v>17320000</v>
+        <v>188410</v>
       </c>
       <c r="E345" s="8" t="n">
-        <v>0.2443</v>
+        <v>0.0501</v>
       </c>
       <c r="F345" s="7" t="n">
-        <v>46.44</v>
-      </c>
-      <c r="G345" s="6" t="inlineStr"/>
+        <v>38.54</v>
+      </c>
+      <c r="G345" s="7" t="n">
+        <v>14.31</v>
+      </c>
       <c r="H345" s="7" t="n">
         <v>1.96</v>
       </c>
       <c r="I345" s="8" t="n">
-        <v>-0.1527</v>
+        <v>0.157</v>
       </c>
       <c r="J345" s="8" t="n">
-        <v>-4.6508</v>
+        <v>-1.2844</v>
       </c>
       <c r="K345" s="6" t="inlineStr">
         <is>
-          <t>Üretici imalatı</t>
+          <t>Dayanıklı olmayan tüketici ürünleri</t>
         </is>
       </c>
       <c r="L345" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST METAL ESYA MAKİNA, BIST ANA, BIST BALIKESİR</t>
+          <t>BIST GIDA ICECEK, BIST TUM-100, BIST SINAI, BIST TÜM, BIST ANA, BIST İZMİR</t>
         </is>
       </c>
       <c r="M345" s="6" t="inlineStr"/>
@@ -15518,42 +15516,42 @@
     <row r="346">
       <c r="A346" s="2" t="inlineStr">
         <is>
-          <t>BRLSM</t>
+          <t>EKOS</t>
         </is>
       </c>
       <c r="B346" s="3" t="n">
-        <v>14.64</v>
+        <v>5.5</v>
       </c>
       <c r="C346" s="4" t="n">
-        <v>-0.0135</v>
+        <v>-0.0248</v>
       </c>
       <c r="D346" s="5" t="n">
-        <v>2870000</v>
+        <v>17320000</v>
       </c>
       <c r="E346" s="4" t="n">
-        <v>0.4823</v>
+        <v>0.2443</v>
       </c>
       <c r="F346" s="3" t="n">
-        <v>44.21</v>
+        <v>46.44</v>
       </c>
       <c r="G346" s="2" t="inlineStr"/>
       <c r="H346" s="3" t="n">
-        <v>1.98</v>
+        <v>1.96</v>
       </c>
       <c r="I346" s="4" t="n">
-        <v>-0.1306</v>
+        <v>-0.1527</v>
       </c>
       <c r="J346" s="4" t="n">
-        <v>-53.3143</v>
+        <v>-4.6508</v>
       </c>
       <c r="K346" s="2" t="inlineStr">
         <is>
-          <t>Enerji-dışı mineraller</t>
+          <t>Üretici imalatı</t>
         </is>
       </c>
       <c r="L346" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST İNŞAAT, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST METAL ESYA MAKİNA, BIST ANA, BIST BALIKESİR</t>
         </is>
       </c>
       <c r="M346" s="2" t="inlineStr"/>
@@ -15561,35 +15559,33 @@
     <row r="347">
       <c r="A347" s="6" t="inlineStr">
         <is>
-          <t>BRSAN</t>
+          <t>BRLSM</t>
         </is>
       </c>
       <c r="B347" s="7" t="n">
-        <v>528</v>
+        <v>14.64</v>
       </c>
       <c r="C347" s="8" t="n">
-        <v>-0.0285</v>
+        <v>-0.0135</v>
       </c>
       <c r="D347" s="9" t="n">
-        <v>1730000</v>
+        <v>2870000</v>
       </c>
       <c r="E347" s="8" t="n">
-        <v>0.1445</v>
+        <v>0.4823</v>
       </c>
       <c r="F347" s="7" t="n">
-        <v>46.65</v>
-      </c>
-      <c r="G347" s="7" t="n">
-        <v>58.86</v>
-      </c>
+        <v>44.21</v>
+      </c>
+      <c r="G347" s="6" t="inlineStr"/>
       <c r="H347" s="7" t="n">
         <v>1.98</v>
       </c>
       <c r="I347" s="8" t="n">
-        <v>0.0375</v>
+        <v>-0.1306</v>
       </c>
       <c r="J347" s="8" t="n">
-        <v>-1.2803</v>
+        <v>-53.3143</v>
       </c>
       <c r="K347" s="6" t="inlineStr">
         <is>
@@ -15598,7 +15594,7 @@
       </c>
       <c r="L347" s="6" t="inlineStr">
         <is>
-          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST SINAI, BIST TÜM, BIST METAL ANA, BIST 50, BIST İSTANBUL, BIST 100-30, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST 50-30, BIST 50-30 AGIRLIK SINIRLAMALI 25, BIST 50-30 AĞIRLIK SINIRLAMALI 10</t>
+          <t>BIST TUM-100, BIST TÜM, BIST İNŞAAT, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
         </is>
       </c>
       <c r="M347" s="6" t="inlineStr"/>
@@ -15606,42 +15602,44 @@
     <row r="348">
       <c r="A348" s="2" t="inlineStr">
         <is>
-          <t>GOODY</t>
+          <t>BRSAN</t>
         </is>
       </c>
       <c r="B348" s="3" t="n">
-        <v>14.96</v>
+        <v>528</v>
       </c>
       <c r="C348" s="4" t="n">
-        <v>-0.0184</v>
+        <v>-0.0285</v>
       </c>
       <c r="D348" s="5" t="n">
-        <v>5950000</v>
+        <v>1730000</v>
       </c>
       <c r="E348" s="4" t="n">
-        <v>0.254</v>
+        <v>0.1445</v>
       </c>
       <c r="F348" s="3" t="n">
-        <v>50.96</v>
-      </c>
-      <c r="G348" s="2" t="inlineStr"/>
+        <v>46.65</v>
+      </c>
+      <c r="G348" s="3" t="n">
+        <v>58.86</v>
+      </c>
       <c r="H348" s="3" t="n">
-        <v>2.02</v>
+        <v>1.98</v>
       </c>
       <c r="I348" s="4" t="n">
-        <v>-1.0324</v>
+        <v>0.0375</v>
       </c>
       <c r="J348" s="4" t="n">
-        <v>-0.2257</v>
+        <v>-1.2803</v>
       </c>
       <c r="K348" s="2" t="inlineStr">
         <is>
-          <t>Dayanıklı tüketim malları</t>
+          <t>Enerji-dışı mineraller</t>
         </is>
       </c>
       <c r="L348" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
+          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST SINAI, BIST TÜM, BIST METAL ANA, BIST 50, BIST İSTANBUL, BIST 100-30, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST 50-30, BIST 50-30 AGIRLIK SINIRLAMALI 25, BIST 50-30 AĞIRLIK SINIRLAMALI 10</t>
         </is>
       </c>
       <c r="M348" s="2" t="inlineStr"/>
@@ -15649,44 +15647,42 @@
     <row r="349">
       <c r="A349" s="6" t="inlineStr">
         <is>
-          <t>TRENJ</t>
+          <t>GOODY</t>
         </is>
       </c>
       <c r="B349" s="7" t="n">
-        <v>96.15000000000001</v>
+        <v>14.96</v>
       </c>
       <c r="C349" s="8" t="n">
-        <v>0.0031</v>
+        <v>-0.0184</v>
       </c>
       <c r="D349" s="9" t="n">
-        <v>1960000</v>
+        <v>5950000</v>
       </c>
       <c r="E349" s="8" t="n">
-        <v>0.3229</v>
+        <v>0.254</v>
       </c>
       <c r="F349" s="7" t="n">
-        <v>46.56</v>
-      </c>
-      <c r="G349" s="7" t="n">
-        <v>110.43</v>
-      </c>
+        <v>50.96</v>
+      </c>
+      <c r="G349" s="6" t="inlineStr"/>
       <c r="H349" s="7" t="n">
         <v>2.02</v>
       </c>
       <c r="I349" s="8" t="n">
-        <v>0.0216</v>
+        <v>-1.0324</v>
       </c>
       <c r="J349" s="8" t="n">
-        <v>-1.4265</v>
+        <v>-0.2257</v>
       </c>
       <c r="K349" s="6" t="inlineStr">
         <is>
-          <t>Enerji mineralleri</t>
+          <t>Dayanıklı tüketim malları</t>
         </is>
       </c>
       <c r="L349" s="6" t="inlineStr">
         <is>
-          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST SINAI, BIST TÜM, BIST MADENCİLİK, BIST 100-30, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST ANKARA</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
         </is>
       </c>
       <c r="M349" s="6" t="inlineStr"/>
@@ -15694,44 +15690,44 @@
     <row r="350">
       <c r="A350" s="2" t="inlineStr">
         <is>
-          <t>ISMEN</t>
+          <t>TRENJ</t>
         </is>
       </c>
       <c r="B350" s="3" t="n">
-        <v>43.62</v>
+        <v>96.15000000000001</v>
       </c>
       <c r="C350" s="4" t="n">
-        <v>0.0111</v>
+        <v>0.0031</v>
       </c>
       <c r="D350" s="5" t="n">
-        <v>11300000</v>
+        <v>1960000</v>
       </c>
       <c r="E350" s="4" t="n">
-        <v>0.3426</v>
+        <v>0.3229</v>
       </c>
       <c r="F350" s="3" t="n">
-        <v>50.72</v>
+        <v>46.56</v>
       </c>
       <c r="G350" s="3" t="n">
-        <v>9.15</v>
+        <v>110.43</v>
       </c>
       <c r="H350" s="3" t="n">
         <v>2.02</v>
       </c>
       <c r="I350" s="4" t="n">
-        <v>0.2423</v>
+        <v>0.0216</v>
       </c>
       <c r="J350" s="4" t="n">
-        <v>0.7472</v>
+        <v>-1.4265</v>
       </c>
       <c r="K350" s="2" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Enerji mineralleri</t>
         </is>
       </c>
       <c r="L350" s="2" t="inlineStr">
         <is>
-          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST MALİ, BIST ARACI KURUMLAR, BIST 100-30, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST TEMETTU 25, BIST TEMETTU, BIST SÜRDÜRÜLEBİLİRLİK</t>
+          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST SINAI, BIST TÜM, BIST MADENCİLİK, BIST 100-30, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST ANKARA</t>
         </is>
       </c>
       <c r="M350" s="2" t="inlineStr"/>
@@ -15739,42 +15735,44 @@
     <row r="351">
       <c r="A351" s="6" t="inlineStr">
         <is>
-          <t>YKSLN</t>
+          <t>ISMEN</t>
         </is>
       </c>
       <c r="B351" s="7" t="n">
-        <v>3.11</v>
+        <v>43.62</v>
       </c>
       <c r="C351" s="8" t="n">
-        <v>-0.0251</v>
+        <v>0.0111</v>
       </c>
       <c r="D351" s="9" t="n">
-        <v>7750000</v>
+        <v>11300000</v>
       </c>
       <c r="E351" s="8" t="n">
-        <v>0.4117</v>
+        <v>0.3426</v>
       </c>
       <c r="F351" s="7" t="n">
-        <v>43.55</v>
-      </c>
-      <c r="G351" s="6" t="inlineStr"/>
+        <v>50.72</v>
+      </c>
+      <c r="G351" s="7" t="n">
+        <v>9.15</v>
+      </c>
       <c r="H351" s="7" t="n">
         <v>2.02</v>
       </c>
       <c r="I351" s="8" t="n">
-        <v>-0.2545</v>
+        <v>0.2423</v>
       </c>
       <c r="J351" s="8" t="n">
-        <v>-0.5023</v>
+        <v>0.7472</v>
       </c>
       <c r="K351" s="6" t="inlineStr">
         <is>
-          <t>Dağıtım servisleri</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L351" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST METAL ANA, BIST İSTANBUL, BIST ANA</t>
+          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST MALİ, BIST ARACI KURUMLAR, BIST 100-30, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST TEMETTU 25, BIST TEMETTU, BIST SÜRDÜRÜLEBİLİRLİK</t>
         </is>
       </c>
       <c r="M351" s="6" t="inlineStr"/>
@@ -15782,44 +15780,42 @@
     <row r="352">
       <c r="A352" s="2" t="inlineStr">
         <is>
-          <t>GARFA</t>
+          <t>YKSLN</t>
         </is>
       </c>
       <c r="B352" s="3" t="n">
-        <v>27.2</v>
+        <v>3.11</v>
       </c>
       <c r="C352" s="4" t="n">
-        <v>-0.0258</v>
+        <v>-0.0251</v>
       </c>
       <c r="D352" s="5" t="n">
-        <v>1010000</v>
+        <v>7750000</v>
       </c>
       <c r="E352" s="4" t="n">
-        <v>0.08380000000000001</v>
+        <v>0.4117</v>
       </c>
       <c r="F352" s="3" t="n">
-        <v>50.9</v>
-      </c>
-      <c r="G352" s="3" t="n">
-        <v>5.08</v>
-      </c>
+        <v>43.55</v>
+      </c>
+      <c r="G352" s="2" t="inlineStr"/>
       <c r="H352" s="3" t="n">
-        <v>2.04</v>
+        <v>2.02</v>
       </c>
       <c r="I352" s="4" t="n">
-        <v>0.5025999999999999</v>
+        <v>-0.2545</v>
       </c>
       <c r="J352" s="4" t="n">
-        <v>-0.121</v>
+        <v>-0.5023</v>
       </c>
       <c r="K352" s="2" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Dağıtım servisleri</t>
         </is>
       </c>
       <c r="L352" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST FIN KIR FAKTÖRIZASYONU, BIST MALİ, BIST ANA, BIST KURUMSAL YÖNETİM</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST METAL ANA, BIST İSTANBUL, BIST ANA</t>
         </is>
       </c>
       <c r="M352" s="2" t="inlineStr"/>
@@ -15827,42 +15823,44 @@
     <row r="353">
       <c r="A353" s="6" t="inlineStr">
         <is>
-          <t>PRZMA</t>
+          <t>GARFA</t>
         </is>
       </c>
       <c r="B353" s="7" t="n">
-        <v>14.15</v>
+        <v>27.2</v>
       </c>
       <c r="C353" s="8" t="n">
-        <v>0.01</v>
+        <v>-0.0258</v>
       </c>
       <c r="D353" s="9" t="n">
-        <v>786080</v>
+        <v>1010000</v>
       </c>
       <c r="E353" s="8" t="n">
-        <v>0.2647</v>
+        <v>0.08380000000000001</v>
       </c>
       <c r="F353" s="7" t="n">
-        <v>46.32</v>
+        <v>50.9</v>
       </c>
       <c r="G353" s="7" t="n">
-        <v>1607.95</v>
+        <v>5.08</v>
       </c>
       <c r="H353" s="7" t="n">
-        <v>2.05</v>
+        <v>2.04</v>
       </c>
       <c r="I353" s="8" t="n">
-        <v>0.0042</v>
-      </c>
-      <c r="J353" s="6" t="inlineStr"/>
+        <v>0.5025999999999999</v>
+      </c>
+      <c r="J353" s="8" t="n">
+        <v>-0.121</v>
+      </c>
       <c r="K353" s="6" t="inlineStr">
         <is>
-          <t>Ticari hizmetler</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L353" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST ORMAN KAĞIT BASIM, BIST İSTANBUL, BIST ANA, BIST KOBİ SANAYİ</t>
+          <t>BIST TUM-100, BIST TÜM, BIST FIN KIR FAKTÖRIZASYONU, BIST MALİ, BIST ANA, BIST KURUMSAL YÖNETİM</t>
         </is>
       </c>
       <c r="M353" s="6" t="inlineStr"/>
@@ -15870,44 +15868,42 @@
     <row r="354">
       <c r="A354" s="2" t="inlineStr">
         <is>
-          <t>DAPGM</t>
+          <t>PRZMA</t>
         </is>
       </c>
       <c r="B354" s="3" t="n">
-        <v>11.37</v>
+        <v>14.15</v>
       </c>
       <c r="C354" s="4" t="n">
-        <v>-0.024</v>
+        <v>0.01</v>
       </c>
       <c r="D354" s="5" t="n">
-        <v>58310000</v>
+        <v>786080</v>
       </c>
       <c r="E354" s="4" t="n">
-        <v>0.2876</v>
+        <v>0.2647</v>
       </c>
       <c r="F354" s="3" t="n">
-        <v>34.31</v>
+        <v>46.32</v>
       </c>
       <c r="G354" s="3" t="n">
-        <v>30.18</v>
+        <v>1607.95</v>
       </c>
       <c r="H354" s="3" t="n">
         <v>2.05</v>
       </c>
       <c r="I354" s="4" t="n">
-        <v>0.0795</v>
-      </c>
-      <c r="J354" s="4" t="n">
-        <v>-0.9063</v>
-      </c>
+        <v>0.0042</v>
+      </c>
+      <c r="J354" s="2" t="inlineStr"/>
       <c r="K354" s="2" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Ticari hizmetler</t>
         </is>
       </c>
       <c r="L354" s="2" t="inlineStr">
         <is>
-          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST İNŞAAT, BIST HİZMETLER, BIST İSTANBUL, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50, BIST KATILIM 30, BIST KATILIM 30 EŞİT AĞIRLIKLI GETİRİ</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST ORMAN KAĞIT BASIM, BIST İSTANBUL, BIST ANA, BIST KOBİ SANAYİ</t>
         </is>
       </c>
       <c r="M354" s="2" t="inlineStr"/>
@@ -15915,44 +15911,44 @@
     <row r="355">
       <c r="A355" s="6" t="inlineStr">
         <is>
-          <t>SEGMN</t>
+          <t>DAPGM</t>
         </is>
       </c>
       <c r="B355" s="7" t="n">
-        <v>58</v>
+        <v>11.37</v>
       </c>
       <c r="C355" s="8" t="n">
-        <v>-0.0153</v>
+        <v>-0.024</v>
       </c>
       <c r="D355" s="9" t="n">
-        <v>4680000</v>
+        <v>58310000</v>
       </c>
       <c r="E355" s="8" t="n">
-        <v>0.2067</v>
+        <v>0.2876</v>
       </c>
       <c r="F355" s="7" t="n">
-        <v>59.23</v>
+        <v>34.31</v>
       </c>
       <c r="G355" s="7" t="n">
-        <v>37.87</v>
+        <v>30.18</v>
       </c>
       <c r="H355" s="7" t="n">
-        <v>2.07</v>
+        <v>2.05</v>
       </c>
       <c r="I355" s="8" t="n">
-        <v>0.0669</v>
+        <v>0.0795</v>
       </c>
       <c r="J355" s="8" t="n">
-        <v>4.7457</v>
+        <v>-0.9063</v>
       </c>
       <c r="K355" s="6" t="inlineStr">
         <is>
-          <t>Dayanıklı olmayan tüketici ürünleri</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L355" s="6" t="inlineStr">
         <is>
-          <t>BIST GIDA ICECEK, BIST TUM-100, BIST SINAI, BIST TÜM, BIST HALKA ARZ, BIST ANA, BIST ANKARA</t>
+          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST İNŞAAT, BIST HİZMETLER, BIST İSTANBUL, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50, BIST KATILIM 30, BIST KATILIM 30 EŞİT AĞIRLIKLI GETİRİ</t>
         </is>
       </c>
       <c r="M355" s="6" t="inlineStr"/>
@@ -15960,44 +15956,44 @@
     <row r="356">
       <c r="A356" s="2" t="inlineStr">
         <is>
-          <t>MAALT</t>
-        </is>
-      </c>
-      <c r="B356" s="5" t="n">
-        <v>1459</v>
+          <t>SEGMN</t>
+        </is>
+      </c>
+      <c r="B356" s="3" t="n">
+        <v>58</v>
       </c>
       <c r="C356" s="4" t="n">
-        <v>0.09949999999999999</v>
+        <v>-0.0153</v>
       </c>
       <c r="D356" s="5" t="n">
-        <v>98280</v>
+        <v>4680000</v>
       </c>
       <c r="E356" s="4" t="n">
-        <v>0.4084</v>
+        <v>0.2067</v>
       </c>
       <c r="F356" s="3" t="n">
-        <v>79.56</v>
+        <v>59.23</v>
       </c>
       <c r="G356" s="3" t="n">
-        <v>340.49</v>
+        <v>37.87</v>
       </c>
       <c r="H356" s="3" t="n">
         <v>2.07</v>
       </c>
       <c r="I356" s="4" t="n">
-        <v>0.008100000000000001</v>
+        <v>0.0669</v>
       </c>
       <c r="J356" s="4" t="n">
-        <v>4.8334</v>
+        <v>4.7457</v>
       </c>
       <c r="K356" s="2" t="inlineStr">
         <is>
-          <t>Tüketici hizmetleri</t>
+          <t>Dayanıklı olmayan tüketici ürünleri</t>
         </is>
       </c>
       <c r="L356" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TURİZM, BIST HİZMETLER, BIST ANA, BIST ANTALYA</t>
+          <t>BIST GIDA ICECEK, BIST TUM-100, BIST SINAI, BIST TÜM, BIST HALKA ARZ, BIST ANA, BIST ANKARA</t>
         </is>
       </c>
       <c r="M356" s="2" t="inlineStr"/>
@@ -16005,40 +16001,44 @@
     <row r="357">
       <c r="A357" s="6" t="inlineStr">
         <is>
-          <t>KNFRT</t>
-        </is>
-      </c>
-      <c r="B357" s="7" t="n">
-        <v>11.5</v>
+          <t>MAALT</t>
+        </is>
+      </c>
+      <c r="B357" s="9" t="n">
+        <v>1459</v>
       </c>
       <c r="C357" s="8" t="n">
-        <v>0.015</v>
+        <v>0.09949999999999999</v>
       </c>
       <c r="D357" s="9" t="n">
-        <v>1880000</v>
+        <v>98280</v>
       </c>
       <c r="E357" s="8" t="n">
-        <v>0.2239</v>
+        <v>0.4084</v>
       </c>
       <c r="F357" s="7" t="n">
-        <v>61.14</v>
-      </c>
-      <c r="G357" s="6" t="inlineStr"/>
+        <v>79.56</v>
+      </c>
+      <c r="G357" s="7" t="n">
+        <v>340.49</v>
+      </c>
       <c r="H357" s="7" t="n">
-        <v>2.08</v>
+        <v>2.07</v>
       </c>
       <c r="I357" s="8" t="n">
-        <v>-0.09710000000000001</v>
-      </c>
-      <c r="J357" s="6" t="inlineStr"/>
+        <v>0.008100000000000001</v>
+      </c>
+      <c r="J357" s="8" t="n">
+        <v>4.8334</v>
+      </c>
       <c r="K357" s="6" t="inlineStr">
         <is>
-          <t>Dayanıklı olmayan tüketici ürünleri</t>
+          <t>Tüketici hizmetleri</t>
         </is>
       </c>
       <c r="L357" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TURİZM, BIST HİZMETLER, BIST ANA, BIST ANTALYA</t>
         </is>
       </c>
       <c r="M357" s="6" t="inlineStr"/>
@@ -16046,42 +16046,40 @@
     <row r="358">
       <c r="A358" s="2" t="inlineStr">
         <is>
-          <t>FENER</t>
+          <t>KNFRT</t>
         </is>
       </c>
       <c r="B358" s="3" t="n">
-        <v>3.03</v>
+        <v>11.5</v>
       </c>
       <c r="C358" s="4" t="n">
-        <v>0.0978</v>
+        <v>0.015</v>
       </c>
       <c r="D358" s="5" t="n">
-        <v>100780000</v>
+        <v>1880000</v>
       </c>
       <c r="E358" s="4" t="n">
-        <v>0.6898000000000001</v>
+        <v>0.2239</v>
       </c>
       <c r="F358" s="3" t="n">
-        <v>60.37</v>
+        <v>61.14</v>
       </c>
       <c r="G358" s="2" t="inlineStr"/>
       <c r="H358" s="3" t="n">
-        <v>2.11</v>
+        <v>2.08</v>
       </c>
       <c r="I358" s="4" t="n">
-        <v>-0.5265</v>
-      </c>
-      <c r="J358" s="4" t="n">
-        <v>-6.582100000000001</v>
-      </c>
+        <v>-0.09710000000000001</v>
+      </c>
+      <c r="J358" s="2" t="inlineStr"/>
       <c r="K358" s="2" t="inlineStr">
         <is>
-          <t>Tüketici hizmetleri</t>
+          <t>Dayanıklı olmayan tüketici ürünleri</t>
         </is>
       </c>
       <c r="L358" s="2" t="inlineStr">
         <is>
-          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST SPOR, BIST HİZMETLER, BIST İSTANBUL, BIST 100-30, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
         </is>
       </c>
       <c r="M358" s="2" t="inlineStr"/>
@@ -16089,42 +16087,42 @@
     <row r="359">
       <c r="A359" s="6" t="inlineStr">
         <is>
-          <t>ACSEL</t>
+          <t>FENER</t>
         </is>
       </c>
       <c r="B359" s="7" t="n">
-        <v>113.7</v>
+        <v>3.03</v>
       </c>
       <c r="C359" s="8" t="n">
-        <v>0.0018</v>
+        <v>0.0978</v>
       </c>
       <c r="D359" s="9" t="n">
-        <v>229470</v>
+        <v>100780000</v>
       </c>
       <c r="E359" s="8" t="n">
-        <v>0.5015999999999999</v>
+        <v>0.6898000000000001</v>
       </c>
       <c r="F359" s="7" t="n">
-        <v>58.02</v>
+        <v>60.37</v>
       </c>
       <c r="G359" s="6" t="inlineStr"/>
       <c r="H359" s="7" t="n">
-        <v>2.12</v>
+        <v>2.11</v>
       </c>
       <c r="I359" s="8" t="n">
-        <v>-0.1212</v>
+        <v>-0.5265</v>
       </c>
       <c r="J359" s="8" t="n">
-        <v>0.7595999999999999</v>
+        <v>-6.582100000000001</v>
       </c>
       <c r="K359" s="6" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
+          <t>Tüketici hizmetleri</t>
         </is>
       </c>
       <c r="L359" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST KATILIM TÜM, BIST ANA, BIST DENİZLİ</t>
+          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST SPOR, BIST HİZMETLER, BIST İSTANBUL, BIST 100-30, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ</t>
         </is>
       </c>
       <c r="M359" s="6" t="inlineStr"/>
@@ -16132,32 +16130,34 @@
     <row r="360">
       <c r="A360" s="2" t="inlineStr">
         <is>
-          <t>AKHAN</t>
+          <t>ACSEL</t>
         </is>
       </c>
       <c r="B360" s="3" t="n">
-        <v>29.12</v>
+        <v>113.7</v>
       </c>
       <c r="C360" s="4" t="n">
-        <v>0.04</v>
+        <v>0.0018</v>
       </c>
       <c r="D360" s="5" t="n">
-        <v>14620000</v>
+        <v>229470</v>
       </c>
       <c r="E360" s="4" t="n">
-        <v>0.2001</v>
+        <v>0.5015999999999999</v>
       </c>
       <c r="F360" s="3" t="n">
-        <v>67.91</v>
+        <v>58.02</v>
       </c>
       <c r="G360" s="2" t="inlineStr"/>
       <c r="H360" s="3" t="n">
-        <v>2.13</v>
+        <v>2.12</v>
       </c>
       <c r="I360" s="4" t="n">
-        <v>0.0438</v>
-      </c>
-      <c r="J360" s="2" t="inlineStr"/>
+        <v>-0.1212</v>
+      </c>
+      <c r="J360" s="4" t="n">
+        <v>0.7595999999999999</v>
+      </c>
       <c r="K360" s="2" t="inlineStr">
         <is>
           <t>İşlenebilen endüstriler</t>
@@ -16165,7 +16165,7 @@
       </c>
       <c r="L360" s="2" t="inlineStr">
         <is>
-          <t>BIST GIDA ICECEK, BIST TUM-100, BIST SINAI, BIST TÜM, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST KATILIM TÜM, BIST ANA, BIST DENİZLİ</t>
         </is>
       </c>
       <c r="M360" s="2" t="inlineStr"/>
@@ -16173,44 +16173,40 @@
     <row r="361">
       <c r="A361" s="6" t="inlineStr">
         <is>
-          <t>GLCVY</t>
+          <t>AKHAN</t>
         </is>
       </c>
       <c r="B361" s="7" t="n">
-        <v>58.75</v>
+        <v>29.12</v>
       </c>
       <c r="C361" s="8" t="n">
-        <v>-0.07480000000000001</v>
+        <v>0.04</v>
       </c>
       <c r="D361" s="9" t="n">
-        <v>1300000</v>
+        <v>14620000</v>
       </c>
       <c r="E361" s="8" t="n">
-        <v>0.189</v>
+        <v>0.2001</v>
       </c>
       <c r="F361" s="7" t="n">
-        <v>31.73</v>
-      </c>
-      <c r="G361" s="7" t="n">
-        <v>5.48</v>
-      </c>
+        <v>67.91</v>
+      </c>
+      <c r="G361" s="6" t="inlineStr"/>
       <c r="H361" s="7" t="n">
         <v>2.13</v>
       </c>
       <c r="I361" s="8" t="n">
-        <v>0.458</v>
-      </c>
-      <c r="J361" s="8" t="n">
-        <v>-0.1093</v>
-      </c>
+        <v>0.0438</v>
+      </c>
+      <c r="J361" s="6" t="inlineStr"/>
       <c r="K361" s="6" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>İşlenebilen endüstriler</t>
         </is>
       </c>
       <c r="L361" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST MALİ, BIST YILDIZ, BIST TEMETTU</t>
+          <t>BIST GIDA ICECEK, BIST TUM-100, BIST SINAI, BIST TÜM, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA</t>
         </is>
       </c>
       <c r="M361" s="6" t="inlineStr"/>
@@ -16218,44 +16214,44 @@
     <row r="362">
       <c r="A362" s="2" t="inlineStr">
         <is>
-          <t>TRMET</t>
+          <t>GLCVY</t>
         </is>
       </c>
       <c r="B362" s="3" t="n">
-        <v>135.2</v>
+        <v>58.75</v>
       </c>
       <c r="C362" s="4" t="n">
-        <v>0.0015</v>
+        <v>-0.07480000000000001</v>
       </c>
       <c r="D362" s="5" t="n">
-        <v>4690000</v>
+        <v>1300000</v>
       </c>
       <c r="E362" s="4" t="n">
-        <v>0.4775</v>
+        <v>0.189</v>
       </c>
       <c r="F362" s="3" t="n">
-        <v>52.22</v>
+        <v>31.73</v>
       </c>
       <c r="G362" s="3" t="n">
-        <v>28.09</v>
+        <v>5.48</v>
       </c>
       <c r="H362" s="3" t="n">
-        <v>2.14</v>
+        <v>2.13</v>
       </c>
       <c r="I362" s="4" t="n">
-        <v>0.09080000000000001</v>
+        <v>0.458</v>
       </c>
       <c r="J362" s="4" t="n">
-        <v>-1.3787</v>
+        <v>-0.1093</v>
       </c>
       <c r="K362" s="2" t="inlineStr">
         <is>
-          <t>Enerji-dışı mineraller</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L362" s="2" t="inlineStr">
         <is>
-          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST SINAI, BIST TÜM, BIST MADENCİLİK, BIST 50, BIST 100-30, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST 50-30, BIST ANKARA, BIST 50-30 AGIRLIK SINIRLAMALI 25, BIST 50-30 AĞIRLIK SINIRLAMALI 10</t>
+          <t>BIST TUM-100, BIST TÜM, BIST MALİ, BIST YILDIZ, BIST TEMETTU</t>
         </is>
       </c>
       <c r="M362" s="2" t="inlineStr"/>
@@ -16263,42 +16259,44 @@
     <row r="363">
       <c r="A363" s="6" t="inlineStr">
         <is>
-          <t>OBAMS</t>
+          <t>TRMET</t>
         </is>
       </c>
       <c r="B363" s="7" t="n">
-        <v>8.17</v>
+        <v>135.2</v>
       </c>
       <c r="C363" s="8" t="n">
-        <v>-0.018</v>
+        <v>0.0015</v>
       </c>
       <c r="D363" s="9" t="n">
-        <v>60150000</v>
+        <v>4690000</v>
       </c>
       <c r="E363" s="8" t="n">
-        <v>0.2611</v>
+        <v>0.4775</v>
       </c>
       <c r="F363" s="7" t="n">
-        <v>48.42</v>
-      </c>
-      <c r="G363" s="6" t="inlineStr"/>
+        <v>52.22</v>
+      </c>
+      <c r="G363" s="7" t="n">
+        <v>28.09</v>
+      </c>
       <c r="H363" s="7" t="n">
         <v>2.14</v>
       </c>
       <c r="I363" s="8" t="n">
-        <v>-0.1977</v>
+        <v>0.09080000000000001</v>
       </c>
       <c r="J363" s="8" t="n">
-        <v>-0.0043</v>
+        <v>-1.3787</v>
       </c>
       <c r="K363" s="6" t="inlineStr">
         <is>
-          <t>Dayanıklı olmayan tüketici ürünleri</t>
+          <t>Enerji-dışı mineraller</t>
         </is>
       </c>
       <c r="L363" s="6" t="inlineStr">
         <is>
-          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST GIDA ICECEK, BIST SINAI, BIST TÜM, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50, BIST KATILIM 30, BIST KATILIM 30 EŞİT AĞIRLIKLI GETİRİ</t>
+          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST SINAI, BIST TÜM, BIST MADENCİLİK, BIST 50, BIST 100-30, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST 50-30, BIST ANKARA, BIST 50-30 AGIRLIK SINIRLAMALI 25, BIST 50-30 AĞIRLIK SINIRLAMALI 10</t>
         </is>
       </c>
       <c r="M363" s="6" t="inlineStr"/>
@@ -16306,44 +16304,42 @@
     <row r="364">
       <c r="A364" s="2" t="inlineStr">
         <is>
-          <t>OFSYM</t>
+          <t>OBAMS</t>
         </is>
       </c>
       <c r="B364" s="3" t="n">
-        <v>60.45</v>
+        <v>8.17</v>
       </c>
       <c r="C364" s="4" t="n">
-        <v>-0.0305</v>
+        <v>-0.018</v>
       </c>
       <c r="D364" s="5" t="n">
-        <v>699820</v>
+        <v>60150000</v>
       </c>
       <c r="E364" s="4" t="n">
-        <v>0.1556</v>
+        <v>0.2611</v>
       </c>
       <c r="F364" s="3" t="n">
-        <v>43.82</v>
-      </c>
-      <c r="G364" s="3" t="n">
-        <v>30.01</v>
-      </c>
+        <v>48.42</v>
+      </c>
+      <c r="G364" s="2" t="inlineStr"/>
       <c r="H364" s="3" t="n">
-        <v>2.15</v>
+        <v>2.14</v>
       </c>
       <c r="I364" s="4" t="n">
-        <v>0.08449999999999999</v>
+        <v>-0.1977</v>
       </c>
       <c r="J364" s="4" t="n">
-        <v>0.1882</v>
+        <v>-0.0043</v>
       </c>
       <c r="K364" s="2" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
+          <t>Dayanıklı olmayan tüketici ürünleri</t>
         </is>
       </c>
       <c r="L364" s="2" t="inlineStr">
         <is>
-          <t>BIST GIDA ICECEK, BIST TUM-100, BIST SINAI, BIST TÜM, BIST KATILIM TÜM, BIST ANA, BIST ANKARA</t>
+          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST GIDA ICECEK, BIST SINAI, BIST TÜM, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50, BIST KATILIM 30, BIST KATILIM 30 EŞİT AĞIRLIKLI GETİRİ</t>
         </is>
       </c>
       <c r="M364" s="2" t="inlineStr"/>
@@ -16351,42 +16347,44 @@
     <row r="365">
       <c r="A365" s="6" t="inlineStr">
         <is>
-          <t>ERSU</t>
+          <t>OFSYM</t>
         </is>
       </c>
       <c r="B365" s="7" t="n">
-        <v>25.68</v>
+        <v>60.45</v>
       </c>
       <c r="C365" s="8" t="n">
-        <v>-0.0418</v>
+        <v>-0.0305</v>
       </c>
       <c r="D365" s="9" t="n">
-        <v>1050000</v>
+        <v>699820</v>
       </c>
       <c r="E365" s="8" t="n">
-        <v>0.7902</v>
+        <v>0.1556</v>
       </c>
       <c r="F365" s="7" t="n">
-        <v>64.36</v>
-      </c>
-      <c r="G365" s="6" t="inlineStr"/>
+        <v>43.82</v>
+      </c>
+      <c r="G365" s="7" t="n">
+        <v>30.01</v>
+      </c>
       <c r="H365" s="7" t="n">
-        <v>2.17</v>
+        <v>2.15</v>
       </c>
       <c r="I365" s="8" t="n">
-        <v>-0.2756</v>
+        <v>0.08449999999999999</v>
       </c>
       <c r="J365" s="8" t="n">
-        <v>0.5871999999999999</v>
+        <v>0.1882</v>
       </c>
       <c r="K365" s="6" t="inlineStr">
         <is>
-          <t>Dayanıklı olmayan tüketici ürünleri</t>
+          <t>İşlenebilen endüstriler</t>
         </is>
       </c>
       <c r="L365" s="6" t="inlineStr">
         <is>
-          <t>BIST GIDA ICECEK, BIST TUM-100, BIST SINAI, BIST TÜM, BIST KOBİ SANAYİ, BIST KONYA</t>
+          <t>BIST GIDA ICECEK, BIST TUM-100, BIST SINAI, BIST TÜM, BIST KATILIM TÜM, BIST ANA, BIST ANKARA</t>
         </is>
       </c>
       <c r="M365" s="6" t="inlineStr"/>
@@ -16394,44 +16392,42 @@
     <row r="366">
       <c r="A366" s="2" t="inlineStr">
         <is>
-          <t>GLYHO</t>
+          <t>ERSU</t>
         </is>
       </c>
       <c r="B366" s="3" t="n">
-        <v>16.06</v>
+        <v>25.68</v>
       </c>
       <c r="C366" s="4" t="n">
-        <v>0.0664</v>
+        <v>-0.0418</v>
       </c>
       <c r="D366" s="5" t="n">
-        <v>8350000</v>
+        <v>1050000</v>
       </c>
       <c r="E366" s="4" t="n">
-        <v>0.645</v>
+        <v>0.7902</v>
       </c>
       <c r="F366" s="3" t="n">
-        <v>61.73</v>
-      </c>
-      <c r="G366" s="3" t="n">
-        <v>6.26</v>
-      </c>
+        <v>64.36</v>
+      </c>
+      <c r="G366" s="2" t="inlineStr"/>
       <c r="H366" s="3" t="n">
-        <v>2.18</v>
+        <v>2.17</v>
       </c>
       <c r="I366" s="4" t="n">
-        <v>0.4401</v>
+        <v>-0.2756</v>
       </c>
       <c r="J366" s="4" t="n">
-        <v>3.6517</v>
+        <v>0.5871999999999999</v>
       </c>
       <c r="K366" s="2" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Dayanıklı olmayan tüketici ürünleri</t>
         </is>
       </c>
       <c r="L366" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HOLDING VE YATIRIM, BIST MALİ, BIST İSTANBUL, BIST YILDIZ, BIST TEMETTU, BIST SÜRDÜRÜLEBİLİRLİK, BIST KURUMSAL YÖNETİM</t>
+          <t>BIST GIDA ICECEK, BIST TUM-100, BIST SINAI, BIST TÜM, BIST KOBİ SANAYİ, BIST KONYA</t>
         </is>
       </c>
       <c r="M366" s="2" t="inlineStr"/>
@@ -16439,44 +16435,44 @@
     <row r="367">
       <c r="A367" s="6" t="inlineStr">
         <is>
-          <t>MTRKS</t>
+          <t>GLYHO</t>
         </is>
       </c>
       <c r="B367" s="7" t="n">
-        <v>21.52</v>
+        <v>16.06</v>
       </c>
       <c r="C367" s="8" t="n">
-        <v>-0.0245</v>
+        <v>0.0664</v>
       </c>
       <c r="D367" s="9" t="n">
-        <v>968830</v>
+        <v>8350000</v>
       </c>
       <c r="E367" s="8" t="n">
-        <v>0.9621</v>
+        <v>0.645</v>
       </c>
       <c r="F367" s="7" t="n">
-        <v>50.89</v>
+        <v>61.73</v>
       </c>
       <c r="G367" s="7" t="n">
-        <v>9.01</v>
+        <v>6.26</v>
       </c>
       <c r="H367" s="7" t="n">
-        <v>2.2</v>
+        <v>2.18</v>
       </c>
       <c r="I367" s="8" t="n">
-        <v>0.3117</v>
+        <v>0.4401</v>
       </c>
       <c r="J367" s="8" t="n">
-        <v>0.7249</v>
+        <v>3.6517</v>
       </c>
       <c r="K367" s="6" t="inlineStr">
         <is>
-          <t>Teknoloji hizmetleri</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L367" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST İSTANBUL, BIST ANA, BIST TEMETTU, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI</t>
+          <t>BIST TUM-100, BIST TÜM, BIST HOLDING VE YATIRIM, BIST MALİ, BIST İSTANBUL, BIST YILDIZ, BIST TEMETTU, BIST SÜRDÜRÜLEBİLİRLİK, BIST KURUMSAL YÖNETİM</t>
         </is>
       </c>
       <c r="M367" s="6" t="inlineStr"/>
@@ -16484,44 +16480,44 @@
     <row r="368">
       <c r="A368" s="2" t="inlineStr">
         <is>
-          <t>BEYAZ</t>
+          <t>MTRKS</t>
         </is>
       </c>
       <c r="B368" s="3" t="n">
-        <v>29.54</v>
+        <v>21.52</v>
       </c>
       <c r="C368" s="4" t="n">
-        <v>-0.018</v>
+        <v>-0.0245</v>
       </c>
       <c r="D368" s="5" t="n">
-        <v>792290</v>
+        <v>968830</v>
       </c>
       <c r="E368" s="4" t="n">
-        <v>0.2455</v>
+        <v>0.9621</v>
       </c>
       <c r="F368" s="3" t="n">
-        <v>56.58</v>
+        <v>50.89</v>
       </c>
       <c r="G368" s="3" t="n">
-        <v>23.11</v>
+        <v>9.01</v>
       </c>
       <c r="H368" s="3" t="n">
-        <v>2.21</v>
+        <v>2.2</v>
       </c>
       <c r="I368" s="4" t="n">
-        <v>0.1128</v>
+        <v>0.3117</v>
       </c>
       <c r="J368" s="4" t="n">
-        <v>-0.9066</v>
+        <v>0.7249</v>
       </c>
       <c r="K368" s="2" t="inlineStr">
         <is>
-          <t>Perakende satış</t>
+          <t>Teknoloji hizmetleri</t>
         </is>
       </c>
       <c r="L368" s="2" t="inlineStr">
         <is>
-          <t>BIST ULASTIRMA, BIST TUM-100, BIST TÜM, BIST HİZMETLER, BIST ANA, BIST BALIKESİR</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST İSTANBUL, BIST ANA, BIST TEMETTU, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI</t>
         </is>
       </c>
       <c r="M368" s="2" t="inlineStr"/>
@@ -16529,42 +16525,44 @@
     <row r="369">
       <c r="A369" s="6" t="inlineStr">
         <is>
-          <t>ADGYO</t>
+          <t>BEYAZ</t>
         </is>
       </c>
       <c r="B369" s="7" t="n">
-        <v>61.7</v>
+        <v>29.54</v>
       </c>
       <c r="C369" s="8" t="n">
-        <v>0.0198</v>
+        <v>-0.018</v>
       </c>
       <c r="D369" s="9" t="n">
-        <v>1130000</v>
+        <v>792290</v>
       </c>
       <c r="E369" s="8" t="n">
-        <v>0.5690999999999999</v>
+        <v>0.2455</v>
       </c>
       <c r="F369" s="7" t="n">
-        <v>61.19</v>
-      </c>
-      <c r="G369" s="6" t="inlineStr"/>
+        <v>56.58</v>
+      </c>
+      <c r="G369" s="7" t="n">
+        <v>23.11</v>
+      </c>
       <c r="H369" s="7" t="n">
         <v>2.21</v>
       </c>
       <c r="I369" s="8" t="n">
-        <v>-0.057</v>
+        <v>0.1128</v>
       </c>
       <c r="J369" s="8" t="n">
-        <v>-19.6193</v>
+        <v>-0.9066</v>
       </c>
       <c r="K369" s="6" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Perakende satış</t>
         </is>
       </c>
       <c r="L369" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST MALİ, BIST YILDIZ</t>
+          <t>BIST ULASTIRMA, BIST TUM-100, BIST TÜM, BIST HİZMETLER, BIST ANA, BIST BALIKESİR</t>
         </is>
       </c>
       <c r="M369" s="6" t="inlineStr"/>
@@ -16572,44 +16570,42 @@
     <row r="370">
       <c r="A370" s="2" t="inlineStr">
         <is>
-          <t>ALVES</t>
+          <t>ADGYO</t>
         </is>
       </c>
       <c r="B370" s="3" t="n">
-        <v>3.76</v>
+        <v>61.7</v>
       </c>
       <c r="C370" s="4" t="n">
-        <v>0.0027</v>
+        <v>0.0198</v>
       </c>
       <c r="D370" s="5" t="n">
-        <v>193770000</v>
+        <v>1130000</v>
       </c>
       <c r="E370" s="4" t="n">
-        <v>0.5014999999999999</v>
+        <v>0.5690999999999999</v>
       </c>
       <c r="F370" s="3" t="n">
-        <v>63.98</v>
-      </c>
-      <c r="G370" s="3" t="n">
-        <v>60.84</v>
-      </c>
+        <v>61.19</v>
+      </c>
+      <c r="G370" s="2" t="inlineStr"/>
       <c r="H370" s="3" t="n">
         <v>2.21</v>
       </c>
       <c r="I370" s="4" t="n">
-        <v>0.04190000000000001</v>
+        <v>-0.057</v>
       </c>
       <c r="J370" s="4" t="n">
-        <v>3.7407</v>
+        <v>-19.6193</v>
       </c>
       <c r="K370" s="2" t="inlineStr">
         <is>
-          <t>Üretici imalatı</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L370" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST METAL ESYA MAKİNA, BIST KATILIM 100, BIST KATILIM TÜM, BIST ANA, BIST ANKARA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST MALİ, BIST YILDIZ</t>
         </is>
       </c>
       <c r="M370" s="2" t="inlineStr"/>
@@ -16617,42 +16613,44 @@
     <row r="371">
       <c r="A371" s="6" t="inlineStr">
         <is>
-          <t>RUZYE</t>
+          <t>ALVES</t>
         </is>
       </c>
       <c r="B371" s="7" t="n">
-        <v>12.11</v>
+        <v>3.76</v>
       </c>
       <c r="C371" s="8" t="n">
-        <v>0.005</v>
+        <v>0.0027</v>
       </c>
       <c r="D371" s="9" t="n">
-        <v>9290000</v>
+        <v>193770000</v>
       </c>
       <c r="E371" s="8" t="n">
-        <v>0.6456000000000001</v>
+        <v>0.5014999999999999</v>
       </c>
       <c r="F371" s="7" t="n">
-        <v>52.76</v>
-      </c>
-      <c r="G371" s="6" t="inlineStr"/>
+        <v>63.98</v>
+      </c>
+      <c r="G371" s="7" t="n">
+        <v>60.84</v>
+      </c>
       <c r="H371" s="7" t="n">
-        <v>2.22</v>
+        <v>2.21</v>
       </c>
       <c r="I371" s="8" t="n">
-        <v>-0.0029</v>
+        <v>0.04190000000000001</v>
       </c>
       <c r="J371" s="8" t="n">
-        <v>-3.8066</v>
+        <v>3.7407</v>
       </c>
       <c r="K371" s="6" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
+          <t>Üretici imalatı</t>
         </is>
       </c>
       <c r="L371" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST MADENCİLİK, BIST ANA, BIST KOBİ SANAYİ, BIST TEKİRDAĞ</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST METAL ESYA MAKİNA, BIST KATILIM 100, BIST KATILIM TÜM, BIST ANA, BIST ANKARA</t>
         </is>
       </c>
       <c r="M371" s="6" t="inlineStr"/>
@@ -16660,42 +16658,42 @@
     <row r="372">
       <c r="A372" s="2" t="inlineStr">
         <is>
-          <t>KLSER</t>
+          <t>RUZYE</t>
         </is>
       </c>
       <c r="B372" s="3" t="n">
-        <v>25.9</v>
+        <v>12.11</v>
       </c>
       <c r="C372" s="4" t="n">
-        <v>-0.0197</v>
+        <v>0.005</v>
       </c>
       <c r="D372" s="5" t="n">
-        <v>1050000</v>
+        <v>9290000</v>
       </c>
       <c r="E372" s="4" t="n">
-        <v>0.2157</v>
+        <v>0.6456000000000001</v>
       </c>
       <c r="F372" s="3" t="n">
-        <v>48.41</v>
+        <v>52.76</v>
       </c>
       <c r="G372" s="2" t="inlineStr"/>
       <c r="H372" s="3" t="n">
-        <v>2.23</v>
+        <v>2.22</v>
       </c>
       <c r="I372" s="4" t="n">
-        <v>-0.5177</v>
+        <v>-0.0029</v>
       </c>
       <c r="J372" s="4" t="n">
-        <v>-2.3054</v>
+        <v>-3.8066</v>
       </c>
       <c r="K372" s="2" t="inlineStr">
         <is>
-          <t>Üretici imalatı</t>
+          <t>İşlenebilen endüstriler</t>
         </is>
       </c>
       <c r="L372" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST TAŞ TOPRAK, BIST YILDIZ, BIST SÜRDÜRÜLEBİLİRLİK, BIST KURUMSAL YÖNETİM</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST MADENCİLİK, BIST ANA, BIST KOBİ SANAYİ, BIST TEKİRDAĞ</t>
         </is>
       </c>
       <c r="M372" s="2" t="inlineStr"/>
@@ -16703,42 +16701,42 @@
     <row r="373">
       <c r="A373" s="6" t="inlineStr">
         <is>
-          <t>KONTR</t>
+          <t>KLSER</t>
         </is>
       </c>
       <c r="B373" s="7" t="n">
-        <v>10.13</v>
+        <v>25.9</v>
       </c>
       <c r="C373" s="8" t="n">
-        <v>0.04650000000000001</v>
+        <v>-0.0197</v>
       </c>
       <c r="D373" s="9" t="n">
-        <v>82560000</v>
+        <v>1050000</v>
       </c>
       <c r="E373" s="8" t="n">
-        <v>0.8695999999999999</v>
+        <v>0.2157</v>
       </c>
       <c r="F373" s="7" t="n">
-        <v>67.05</v>
+        <v>48.41</v>
       </c>
       <c r="G373" s="6" t="inlineStr"/>
       <c r="H373" s="7" t="n">
-        <v>2.25</v>
+        <v>2.23</v>
       </c>
       <c r="I373" s="8" t="n">
-        <v>-0.213</v>
+        <v>-0.5177</v>
       </c>
       <c r="J373" s="8" t="n">
-        <v>0.5029</v>
+        <v>-2.3054</v>
       </c>
       <c r="K373" s="6" t="inlineStr">
         <is>
-          <t>Elektrik, Su, Gaz Hizmetleri</t>
+          <t>Üretici imalatı</t>
         </is>
       </c>
       <c r="L373" s="6" t="inlineStr">
         <is>
-          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST 50, BIST HİZMETLER, BIST İSTANBUL, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50, BIST SÜRDÜRÜLEBİLİRLİK, BIST KURUMSAL YÖNETİM, BIST KATILIM 30, BIST 50-30, BIST KATILIM SÜRDÜRÜLEBİLİRLİİK, BIST KATILIM 30 EŞİT AĞIRLIKLI GETİRİ, BIST 50-30 AGIRLIK SINIRLAMALI 25, BIST 50-30 AĞIRLIK SINIRLAMALI 10</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST TAŞ TOPRAK, BIST YILDIZ, BIST SÜRDÜRÜLEBİLİRLİK, BIST KURUMSAL YÖNETİM</t>
         </is>
       </c>
       <c r="M373" s="6" t="inlineStr"/>
@@ -16746,44 +16744,42 @@
     <row r="374">
       <c r="A374" s="2" t="inlineStr">
         <is>
-          <t>SUNTK</t>
+          <t>KONTR</t>
         </is>
       </c>
       <c r="B374" s="3" t="n">
-        <v>33.76</v>
+        <v>10.13</v>
       </c>
       <c r="C374" s="4" t="n">
-        <v>-0.0463</v>
+        <v>0.04650000000000001</v>
       </c>
       <c r="D374" s="5" t="n">
-        <v>1090000</v>
+        <v>82560000</v>
       </c>
       <c r="E374" s="4" t="n">
-        <v>0.2071</v>
+        <v>0.8695999999999999</v>
       </c>
       <c r="F374" s="3" t="n">
-        <v>42.94</v>
-      </c>
-      <c r="G374" s="3" t="n">
-        <v>23.65</v>
-      </c>
+        <v>67.05</v>
+      </c>
+      <c r="G374" s="2" t="inlineStr"/>
       <c r="H374" s="3" t="n">
-        <v>2.27</v>
+        <v>2.25</v>
       </c>
       <c r="I374" s="4" t="n">
-        <v>0.1095</v>
+        <v>-0.213</v>
       </c>
       <c r="J374" s="4" t="n">
-        <v>-0.2312</v>
+        <v>0.5029</v>
       </c>
       <c r="K374" s="2" t="inlineStr">
         <is>
-          <t>Dayanıklı olmayan tüketici ürünleri</t>
+          <t>Elektrik, Su, Gaz Hizmetleri</t>
         </is>
       </c>
       <c r="L374" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST TEKSTİL DERİ, BIST KATILIM 100, BIST KATILIM TÜM, BIST YILDIZ, BIST TEMETTU, BIST SÜRDÜRÜLEBİLİRLİK, BIST KURUMSAL YÖNETİM, BIST KATILIM TEMETTU, BIST İZMİR, BIST KATILIM SÜRDÜRÜLEBİLİRLİİK</t>
+          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST 50, BIST HİZMETLER, BIST İSTANBUL, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50, BIST SÜRDÜRÜLEBİLİRLİK, BIST KURUMSAL YÖNETİM, BIST KATILIM 30, BIST 50-30, BIST KATILIM SÜRDÜRÜLEBİLİRLİİK, BIST KATILIM 30 EŞİT AĞIRLIKLI GETİRİ, BIST 50-30 AGIRLIK SINIRLAMALI 25, BIST 50-30 AĞIRLIK SINIRLAMALI 10</t>
         </is>
       </c>
       <c r="M374" s="2" t="inlineStr"/>
@@ -16791,40 +16787,44 @@
     <row r="375">
       <c r="A375" s="6" t="inlineStr">
         <is>
-          <t>DESPC</t>
+          <t>SUNTK</t>
         </is>
       </c>
       <c r="B375" s="7" t="n">
-        <v>39.96</v>
+        <v>33.76</v>
       </c>
       <c r="C375" s="8" t="n">
-        <v>-0.0287</v>
+        <v>-0.0463</v>
       </c>
       <c r="D375" s="9" t="n">
-        <v>491660</v>
-      </c>
-      <c r="E375" s="6" t="inlineStr"/>
+        <v>1090000</v>
+      </c>
+      <c r="E375" s="8" t="n">
+        <v>0.2071</v>
+      </c>
       <c r="F375" s="7" t="n">
-        <v>49.52</v>
-      </c>
-      <c r="G375" s="6" t="inlineStr"/>
+        <v>42.94</v>
+      </c>
+      <c r="G375" s="7" t="n">
+        <v>23.65</v>
+      </c>
       <c r="H375" s="7" t="n">
         <v>2.27</v>
       </c>
       <c r="I375" s="8" t="n">
-        <v>-0.1176</v>
+        <v>0.1095</v>
       </c>
       <c r="J375" s="8" t="n">
-        <v>-19.3798</v>
+        <v>-0.2312</v>
       </c>
       <c r="K375" s="6" t="inlineStr">
         <is>
-          <t>Dağıtım servisleri</t>
+          <t>Dayanıklı olmayan tüketici ürünleri</t>
         </is>
       </c>
       <c r="L375" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST TEKSTİL DERİ, BIST KATILIM 100, BIST KATILIM TÜM, BIST YILDIZ, BIST TEMETTU, BIST SÜRDÜRÜLEBİLİRLİK, BIST KURUMSAL YÖNETİM, BIST KATILIM TEMETTU, BIST İZMİR, BIST KATILIM SÜRDÜRÜLEBİLİRLİİK</t>
         </is>
       </c>
       <c r="M375" s="6" t="inlineStr"/>
@@ -16832,42 +16832,40 @@
     <row r="376">
       <c r="A376" s="2" t="inlineStr">
         <is>
-          <t>EGEEN</t>
-        </is>
-      </c>
-      <c r="B376" s="5" t="n">
-        <v>5655</v>
+          <t>DESPC</t>
+        </is>
+      </c>
+      <c r="B376" s="3" t="n">
+        <v>39.96</v>
       </c>
       <c r="C376" s="4" t="n">
-        <v>-0.0144</v>
+        <v>-0.0287</v>
       </c>
       <c r="D376" s="5" t="n">
-        <v>12050</v>
-      </c>
-      <c r="E376" s="4" t="n">
-        <v>0.3637</v>
-      </c>
+        <v>491660</v>
+      </c>
+      <c r="E376" s="2" t="inlineStr"/>
       <c r="F376" s="3" t="n">
-        <v>43.67</v>
+        <v>49.52</v>
       </c>
       <c r="G376" s="2" t="inlineStr"/>
       <c r="H376" s="3" t="n">
-        <v>2.28</v>
+        <v>2.27</v>
       </c>
       <c r="I376" s="4" t="n">
-        <v>-0.0145</v>
+        <v>-0.1176</v>
       </c>
       <c r="J376" s="4" t="n">
-        <v>-13.2704</v>
+        <v>-19.3798</v>
       </c>
       <c r="K376" s="2" t="inlineStr">
         <is>
-          <t>Üretici imalatı</t>
+          <t>Dağıtım servisleri</t>
         </is>
       </c>
       <c r="L376" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST METAL ESYA MAKİNA, BIST YILDIZ, BIST TEMETTU, BIST İZMİR</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI</t>
         </is>
       </c>
       <c r="M376" s="2" t="inlineStr"/>
@@ -16875,44 +16873,42 @@
     <row r="377">
       <c r="A377" s="6" t="inlineStr">
         <is>
-          <t>LMKDC</t>
-        </is>
-      </c>
-      <c r="B377" s="7" t="n">
-        <v>33.7</v>
+          <t>EGEEN</t>
+        </is>
+      </c>
+      <c r="B377" s="9" t="n">
+        <v>5655</v>
       </c>
       <c r="C377" s="8" t="n">
-        <v>0.0421</v>
+        <v>-0.0144</v>
       </c>
       <c r="D377" s="9" t="n">
-        <v>6280000</v>
+        <v>12050</v>
       </c>
       <c r="E377" s="8" t="n">
-        <v>0.3021</v>
+        <v>0.3637</v>
       </c>
       <c r="F377" s="7" t="n">
-        <v>59.98</v>
-      </c>
-      <c r="G377" s="7" t="n">
-        <v>8.92</v>
-      </c>
+        <v>43.67</v>
+      </c>
+      <c r="G377" s="6" t="inlineStr"/>
       <c r="H377" s="7" t="n">
-        <v>2.3</v>
+        <v>2.28</v>
       </c>
       <c r="I377" s="8" t="n">
-        <v>0.3184</v>
+        <v>-0.0145</v>
       </c>
       <c r="J377" s="8" t="n">
-        <v>-0.1897</v>
+        <v>-13.2704</v>
       </c>
       <c r="K377" s="6" t="inlineStr">
         <is>
-          <t>Enerji-dışı mineraller</t>
+          <t>Üretici imalatı</t>
         </is>
       </c>
       <c r="L377" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST TAŞ TOPRAK, BIST KATILIM 100, BIST KATILIM TÜM, BIST YILDIZ, BIST KATILIM 50</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST METAL ESYA MAKİNA, BIST YILDIZ, BIST TEMETTU, BIST İZMİR</t>
         </is>
       </c>
       <c r="M377" s="6" t="inlineStr"/>
@@ -16920,44 +16916,44 @@
     <row r="378">
       <c r="A378" s="2" t="inlineStr">
         <is>
-          <t>EBEBK</t>
+          <t>LMKDC</t>
         </is>
       </c>
       <c r="B378" s="3" t="n">
-        <v>66.3</v>
+        <v>33.7</v>
       </c>
       <c r="C378" s="4" t="n">
-        <v>0.02</v>
+        <v>0.0421</v>
       </c>
       <c r="D378" s="5" t="n">
-        <v>693930</v>
+        <v>6280000</v>
       </c>
       <c r="E378" s="4" t="n">
-        <v>0.253</v>
+        <v>0.3021</v>
       </c>
       <c r="F378" s="3" t="n">
-        <v>64.22</v>
+        <v>59.98</v>
       </c>
       <c r="G378" s="3" t="n">
-        <v>167.64</v>
+        <v>8.92</v>
       </c>
       <c r="H378" s="3" t="n">
-        <v>2.32</v>
+        <v>2.3</v>
       </c>
       <c r="I378" s="4" t="n">
-        <v>0.0154</v>
+        <v>0.3184</v>
       </c>
       <c r="J378" s="4" t="n">
-        <v>-0.8693000000000001</v>
+        <v>-0.1897</v>
       </c>
       <c r="K378" s="2" t="inlineStr">
         <is>
-          <t>Perakende satış</t>
+          <t>Enerji-dışı mineraller</t>
         </is>
       </c>
       <c r="L378" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST KATILIM TÜM, BIST YILDIZ</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST TAŞ TOPRAK, BIST KATILIM 100, BIST KATILIM TÜM, BIST YILDIZ, BIST KATILIM 50</t>
         </is>
       </c>
       <c r="M378" s="2" t="inlineStr"/>
@@ -16965,42 +16961,44 @@
     <row r="379">
       <c r="A379" s="6" t="inlineStr">
         <is>
-          <t>SONME</t>
+          <t>EBEBK</t>
         </is>
       </c>
       <c r="B379" s="7" t="n">
-        <v>136.9</v>
+        <v>66.3</v>
       </c>
       <c r="C379" s="8" t="n">
-        <v>-0.0165</v>
+        <v>0.02</v>
       </c>
       <c r="D379" s="9" t="n">
-        <v>29690</v>
+        <v>693930</v>
       </c>
       <c r="E379" s="8" t="n">
-        <v>0.0789</v>
+        <v>0.253</v>
       </c>
       <c r="F379" s="7" t="n">
-        <v>37.31</v>
-      </c>
-      <c r="G379" s="6" t="inlineStr"/>
+        <v>64.22</v>
+      </c>
+      <c r="G379" s="7" t="n">
+        <v>167.64</v>
+      </c>
       <c r="H379" s="7" t="n">
-        <v>2.33</v>
+        <v>2.32</v>
       </c>
       <c r="I379" s="8" t="n">
-        <v>-0.057</v>
+        <v>0.0154</v>
       </c>
       <c r="J379" s="8" t="n">
-        <v>-22.838</v>
+        <v>-0.8693000000000001</v>
       </c>
       <c r="K379" s="6" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
+          <t>Perakende satış</t>
         </is>
       </c>
       <c r="L379" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HİZMETLER, BIST BURSA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST KATILIM TÜM, BIST YILDIZ</t>
         </is>
       </c>
       <c r="M379" s="6" t="inlineStr"/>
@@ -17008,42 +17006,42 @@
     <row r="380">
       <c r="A380" s="2" t="inlineStr">
         <is>
-          <t>BYDNR</t>
+          <t>SONME</t>
         </is>
       </c>
       <c r="B380" s="3" t="n">
-        <v>40.88</v>
+        <v>136.9</v>
       </c>
       <c r="C380" s="4" t="n">
-        <v>-0.0024</v>
+        <v>-0.0165</v>
       </c>
       <c r="D380" s="5" t="n">
-        <v>672460</v>
+        <v>29690</v>
       </c>
       <c r="E380" s="4" t="n">
-        <v>0.1667</v>
+        <v>0.0789</v>
       </c>
       <c r="F380" s="3" t="n">
-        <v>58.97</v>
+        <v>37.31</v>
       </c>
       <c r="G380" s="2" t="inlineStr"/>
       <c r="H380" s="3" t="n">
-        <v>2.34</v>
+        <v>2.33</v>
       </c>
       <c r="I380" s="4" t="n">
-        <v>-0.0684</v>
+        <v>-0.057</v>
       </c>
       <c r="J380" s="4" t="n">
-        <v>-1.9324</v>
+        <v>-22.838</v>
       </c>
       <c r="K380" s="2" t="inlineStr">
         <is>
-          <t>Tüketici hizmetleri</t>
+          <t>İşlenebilen endüstriler</t>
         </is>
       </c>
       <c r="L380" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TURİZM, BIST HİZMETLER, BIST ANA, BIST İZMİR</t>
+          <t>BIST TUM-100, BIST TÜM, BIST HİZMETLER, BIST BURSA</t>
         </is>
       </c>
       <c r="M380" s="2" t="inlineStr"/>
@@ -17051,44 +17049,42 @@
     <row r="381">
       <c r="A381" s="6" t="inlineStr">
         <is>
-          <t>FROTO</t>
+          <t>BYDNR</t>
         </is>
       </c>
       <c r="B381" s="7" t="n">
-        <v>104.9</v>
+        <v>40.88</v>
       </c>
       <c r="C381" s="8" t="n">
-        <v>-0.0038</v>
+        <v>-0.0024</v>
       </c>
       <c r="D381" s="9" t="n">
-        <v>15030000</v>
+        <v>672460</v>
       </c>
       <c r="E381" s="8" t="n">
-        <v>0.1789</v>
+        <v>0.1667</v>
       </c>
       <c r="F381" s="7" t="n">
-        <v>49.49</v>
-      </c>
-      <c r="G381" s="7" t="n">
-        <v>11.28</v>
-      </c>
+        <v>58.97</v>
+      </c>
+      <c r="G381" s="6" t="inlineStr"/>
       <c r="H381" s="7" t="n">
-        <v>2.36</v>
+        <v>2.34</v>
       </c>
       <c r="I381" s="8" t="n">
-        <v>0.2405</v>
+        <v>-0.0684</v>
       </c>
       <c r="J381" s="8" t="n">
-        <v>0.3834</v>
+        <v>-1.9324</v>
       </c>
       <c r="K381" s="6" t="inlineStr">
         <is>
-          <t>Dayanıklı tüketim malları</t>
+          <t>Tüketici hizmetleri</t>
         </is>
       </c>
       <c r="L381" s="6" t="inlineStr">
         <is>
-          <t>BIST 100, BIST 30, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST SINAI, BIST TÜM, BIST 50, BIST METAL ESYA MAKİNA, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST TEMETTU 25, BIST TEMETTU, BIST SÜRDÜRÜLEBİLİRLİK, BIST KURUMSAL YÖNETİM, BIST KOCAELI, BIST 30 AĞIRLIK SINIRLAMALI 10, BIST 30 EŞİT AĞIRLIKLI GETİRİ, BIST 30 AĞIRLIK SINIRLAMALI 25, STOXX Emerging Markets 1500</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TURİZM, BIST HİZMETLER, BIST ANA, BIST İZMİR</t>
         </is>
       </c>
       <c r="M381" s="6" t="inlineStr"/>
@@ -17096,44 +17092,44 @@
     <row r="382">
       <c r="A382" s="2" t="inlineStr">
         <is>
-          <t>MOPAS</t>
+          <t>FROTO</t>
         </is>
       </c>
       <c r="B382" s="3" t="n">
-        <v>42</v>
+        <v>104.9</v>
       </c>
       <c r="C382" s="4" t="n">
-        <v>0.012</v>
+        <v>-0.0038</v>
       </c>
       <c r="D382" s="5" t="n">
-        <v>7200000</v>
+        <v>15030000</v>
       </c>
       <c r="E382" s="4" t="n">
-        <v>0.21</v>
+        <v>0.1789</v>
       </c>
       <c r="F382" s="3" t="n">
-        <v>47.35</v>
+        <v>49.49</v>
       </c>
       <c r="G382" s="3" t="n">
-        <v>48.5</v>
+        <v>11.28</v>
       </c>
       <c r="H382" s="3" t="n">
         <v>2.36</v>
       </c>
       <c r="I382" s="4" t="n">
-        <v>0.0633</v>
+        <v>0.2405</v>
       </c>
       <c r="J382" s="4" t="n">
-        <v>-0.2432</v>
+        <v>0.3834</v>
       </c>
       <c r="K382" s="2" t="inlineStr">
         <is>
-          <t>Perakende satış</t>
+          <t>Dayanıklı tüketim malları</t>
         </is>
       </c>
       <c r="L382" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST TİCARET, BIST HİZMETLER, BIST YILDIZ</t>
+          <t>BIST 100, BIST 30, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST SINAI, BIST TÜM, BIST 50, BIST METAL ESYA MAKİNA, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST TEMETTU 25, BIST TEMETTU, BIST SÜRDÜRÜLEBİLİRLİK, BIST KURUMSAL YÖNETİM, BIST KOCAELI, BIST 30 AĞIRLIK SINIRLAMALI 10, BIST 30 EŞİT AĞIRLIKLI GETİRİ, BIST 30 AĞIRLIK SINIRLAMALI 25, STOXX Emerging Markets 1500</t>
         </is>
       </c>
       <c r="M382" s="2" t="inlineStr"/>
@@ -17141,44 +17137,44 @@
     <row r="383">
       <c r="A383" s="6" t="inlineStr">
         <is>
-          <t>TOASO</t>
+          <t>MOPAS</t>
         </is>
       </c>
       <c r="B383" s="7" t="n">
-        <v>283.75</v>
+        <v>42</v>
       </c>
       <c r="C383" s="8" t="n">
-        <v>-0.0035</v>
+        <v>0.012</v>
       </c>
       <c r="D383" s="9" t="n">
-        <v>3300000</v>
+        <v>7200000</v>
       </c>
       <c r="E383" s="8" t="n">
-        <v>0.2429</v>
+        <v>0.21</v>
       </c>
       <c r="F383" s="7" t="n">
-        <v>49.63</v>
+        <v>47.35</v>
       </c>
       <c r="G383" s="7" t="n">
-        <v>17.21</v>
+        <v>48.5</v>
       </c>
       <c r="H383" s="7" t="n">
         <v>2.36</v>
       </c>
       <c r="I383" s="8" t="n">
-        <v>0.1539</v>
+        <v>0.0633</v>
       </c>
       <c r="J383" s="8" t="n">
-        <v>3.4881</v>
+        <v>-0.2432</v>
       </c>
       <c r="K383" s="6" t="inlineStr">
         <is>
-          <t>Dayanıklı tüketim malları</t>
+          <t>Perakende satış</t>
         </is>
       </c>
       <c r="L383" s="6" t="inlineStr">
         <is>
-          <t>BIST 100, BIST 30, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST SINAI, BIST TÜM, BIST 50, BIST METAL ESYA MAKİNA, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST TEMETTU 25, BIST TEMETTU, BIST SÜRDÜRÜLEBİLİRLİK, BIST KURUMSAL YÖNETİM, BIST BURSA, BIST 30 AĞIRLIK SINIRLAMALI 10, BIST 30 EŞİT AĞIRLIKLI GETİRİ, BIST 30 AĞIRLIK SINIRLAMALI 25</t>
+          <t>BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST TİCARET, BIST HİZMETLER, BIST YILDIZ</t>
         </is>
       </c>
       <c r="M383" s="6" t="inlineStr"/>
@@ -17186,40 +17182,44 @@
     <row r="384">
       <c r="A384" s="2" t="inlineStr">
         <is>
-          <t>SMART</t>
+          <t>TOASO</t>
         </is>
       </c>
       <c r="B384" s="3" t="n">
-        <v>31.74</v>
+        <v>283.75</v>
       </c>
       <c r="C384" s="4" t="n">
-        <v>-0.03700000000000001</v>
+        <v>-0.0035</v>
       </c>
       <c r="D384" s="5" t="n">
-        <v>4130000</v>
-      </c>
-      <c r="E384" s="2" t="inlineStr"/>
+        <v>3300000</v>
+      </c>
+      <c r="E384" s="4" t="n">
+        <v>0.2429</v>
+      </c>
       <c r="F384" s="3" t="n">
-        <v>48.42</v>
-      </c>
-      <c r="G384" s="2" t="inlineStr"/>
+        <v>49.63</v>
+      </c>
+      <c r="G384" s="3" t="n">
+        <v>17.21</v>
+      </c>
       <c r="H384" s="3" t="n">
-        <v>2.37</v>
+        <v>2.36</v>
       </c>
       <c r="I384" s="4" t="n">
-        <v>-0.0582</v>
+        <v>0.1539</v>
       </c>
       <c r="J384" s="4" t="n">
-        <v>-15.5087</v>
+        <v>3.4881</v>
       </c>
       <c r="K384" s="2" t="inlineStr">
         <is>
-          <t>Teknoloji hizmetleri</t>
+          <t>Dayanıklı tüketim malları</t>
         </is>
       </c>
       <c r="L384" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI</t>
+          <t>BIST 100, BIST 30, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST SINAI, BIST TÜM, BIST 50, BIST METAL ESYA MAKİNA, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST TEMETTU 25, BIST TEMETTU, BIST SÜRDÜRÜLEBİLİRLİK, BIST KURUMSAL YÖNETİM, BIST BURSA, BIST 30 AĞIRLIK SINIRLAMALI 10, BIST 30 EŞİT AĞIRLIKLI GETİRİ, BIST 30 AĞIRLIK SINIRLAMALI 25</t>
         </is>
       </c>
       <c r="M384" s="2" t="inlineStr"/>
@@ -17227,34 +17227,32 @@
     <row r="385">
       <c r="A385" s="6" t="inlineStr">
         <is>
-          <t>OBASE</t>
+          <t>SMART</t>
         </is>
       </c>
       <c r="B385" s="7" t="n">
-        <v>37.44</v>
+        <v>31.74</v>
       </c>
       <c r="C385" s="8" t="n">
-        <v>0.006500000000000001</v>
+        <v>-0.03700000000000001</v>
       </c>
       <c r="D385" s="9" t="n">
-        <v>637670</v>
-      </c>
-      <c r="E385" s="8" t="n">
-        <v>0.328</v>
-      </c>
+        <v>4130000</v>
+      </c>
+      <c r="E385" s="6" t="inlineStr"/>
       <c r="F385" s="7" t="n">
-        <v>63.46</v>
-      </c>
-      <c r="G385" s="7" t="n">
-        <v>237.56</v>
-      </c>
+        <v>48.42</v>
+      </c>
+      <c r="G385" s="6" t="inlineStr"/>
       <c r="H385" s="7" t="n">
-        <v>2.4</v>
+        <v>2.37</v>
       </c>
       <c r="I385" s="8" t="n">
-        <v>0.0114</v>
-      </c>
-      <c r="J385" s="6" t="inlineStr"/>
+        <v>-0.0582</v>
+      </c>
+      <c r="J385" s="8" t="n">
+        <v>-15.5087</v>
+      </c>
       <c r="K385" s="6" t="inlineStr">
         <is>
           <t>Teknoloji hizmetleri</t>
@@ -17270,44 +17268,42 @@
     <row r="386">
       <c r="A386" s="2" t="inlineStr">
         <is>
-          <t>SARKY</t>
+          <t>OBASE</t>
         </is>
       </c>
       <c r="B386" s="3" t="n">
-        <v>27.96</v>
+        <v>37.44</v>
       </c>
       <c r="C386" s="4" t="n">
-        <v>-0.0043</v>
+        <v>0.006500000000000001</v>
       </c>
       <c r="D386" s="5" t="n">
-        <v>10090000</v>
+        <v>637670</v>
       </c>
       <c r="E386" s="4" t="n">
-        <v>0.6587000000000001</v>
+        <v>0.328</v>
       </c>
       <c r="F386" s="3" t="n">
-        <v>44.18</v>
+        <v>63.46</v>
       </c>
       <c r="G386" s="3" t="n">
-        <v>106.23</v>
+        <v>237.56</v>
       </c>
       <c r="H386" s="3" t="n">
-        <v>2.42</v>
+        <v>2.4</v>
       </c>
       <c r="I386" s="4" t="n">
-        <v>0.0294</v>
-      </c>
-      <c r="J386" s="4" t="n">
-        <v>-2.2136</v>
-      </c>
+        <v>0.0114</v>
+      </c>
+      <c r="J386" s="2" t="inlineStr"/>
       <c r="K386" s="2" t="inlineStr">
         <is>
-          <t>Üretici imalatı</t>
+          <t>Teknoloji hizmetleri</t>
         </is>
       </c>
       <c r="L386" s="2" t="inlineStr">
         <is>
-          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST SINAI, BIST TÜM, BIST METAL ANA, BIST 100-30, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST TEMETTU, BIST KATILIM TEMETTU, BIST KOCAELI</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI</t>
         </is>
       </c>
       <c r="M386" s="2" t="inlineStr"/>
@@ -17315,42 +17311,44 @@
     <row r="387">
       <c r="A387" s="6" t="inlineStr">
         <is>
-          <t>CEOEM</t>
+          <t>SARKY</t>
         </is>
       </c>
       <c r="B387" s="7" t="n">
-        <v>24.04</v>
+        <v>27.96</v>
       </c>
       <c r="C387" s="8" t="n">
-        <v>0.0092</v>
+        <v>-0.0043</v>
       </c>
       <c r="D387" s="9" t="n">
-        <v>3140000</v>
-      </c>
-      <c r="E387" s="6" t="inlineStr"/>
+        <v>10090000</v>
+      </c>
+      <c r="E387" s="8" t="n">
+        <v>0.6587000000000001</v>
+      </c>
       <c r="F387" s="7" t="n">
-        <v>61.01</v>
+        <v>44.18</v>
       </c>
       <c r="G387" s="7" t="n">
-        <v>372.71</v>
+        <v>106.23</v>
       </c>
       <c r="H387" s="7" t="n">
         <v>2.42</v>
       </c>
       <c r="I387" s="8" t="n">
-        <v>0.0073</v>
+        <v>0.0294</v>
       </c>
       <c r="J387" s="8" t="n">
-        <v>-0.3059</v>
+        <v>-2.2136</v>
       </c>
       <c r="K387" s="6" t="inlineStr">
         <is>
-          <t>Tüketici hizmetleri</t>
+          <t>Üretici imalatı</t>
         </is>
       </c>
       <c r="L387" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HİZMETLER, BIST İSTANBUL, BIST ANA</t>
+          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST SINAI, BIST TÜM, BIST METAL ANA, BIST 100-30, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST TEMETTU, BIST KATILIM TEMETTU, BIST KOCAELI</t>
         </is>
       </c>
       <c r="M387" s="6" t="inlineStr"/>
@@ -17358,44 +17356,42 @@
     <row r="388">
       <c r="A388" s="2" t="inlineStr">
         <is>
-          <t>MAVI</t>
+          <t>CEOEM</t>
         </is>
       </c>
       <c r="B388" s="3" t="n">
-        <v>43.18</v>
+        <v>24.04</v>
       </c>
       <c r="C388" s="4" t="n">
-        <v>-0.0074</v>
+        <v>0.0092</v>
       </c>
       <c r="D388" s="5" t="n">
-        <v>6620000</v>
-      </c>
-      <c r="E388" s="4" t="n">
-        <v>0.7259</v>
-      </c>
+        <v>3140000</v>
+      </c>
+      <c r="E388" s="2" t="inlineStr"/>
       <c r="F388" s="3" t="n">
-        <v>51.43</v>
+        <v>61.01</v>
       </c>
       <c r="G388" s="3" t="n">
-        <v>15.76</v>
+        <v>372.71</v>
       </c>
       <c r="H388" s="3" t="n">
-        <v>2.44</v>
+        <v>2.42</v>
       </c>
       <c r="I388" s="4" t="n">
-        <v>0.1794</v>
+        <v>0.0073</v>
       </c>
       <c r="J388" s="4" t="n">
-        <v>-0.9131999999999999</v>
+        <v>-0.3059</v>
       </c>
       <c r="K388" s="2" t="inlineStr">
         <is>
-          <t>Dayanıklı olmayan tüketici ürünleri</t>
+          <t>Tüketici hizmetleri</t>
         </is>
       </c>
       <c r="L388" s="2" t="inlineStr">
         <is>
-          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST 50, BIST TİCARET, BIST HİZMETLER, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST TEMETTU 25, BIST TEMETTU, BIST KATILIM 50, BIST SÜRDÜRÜLEBİLİRLİK, BIST KATILIM 30, BIST 50-30, BIST KATILIM TEMETTU, BIST SÜRDÜRÜLEBİLİRLİK 25, BIST KATILIM SÜRDÜRÜLEBİLİRLİİK, BIST KATILIM 30 EŞİT AĞIRLIKLI GETİRİ, BIST 50-30 AGIRLIK SINIRLAMALI 25, BIST 50-30 AĞIRLIK SINIRLAMALI 10</t>
+          <t>BIST TUM-100, BIST TÜM, BIST HİZMETLER, BIST İSTANBUL, BIST ANA</t>
         </is>
       </c>
       <c r="M388" s="2" t="inlineStr"/>
@@ -17403,33 +17399,35 @@
     <row r="389">
       <c r="A389" s="6" t="inlineStr">
         <is>
-          <t>DUNYH</t>
+          <t>MAVI</t>
         </is>
       </c>
       <c r="B389" s="7" t="n">
-        <v>106</v>
+        <v>43.18</v>
       </c>
       <c r="C389" s="8" t="n">
-        <v>-0.0594</v>
+        <v>-0.0074</v>
       </c>
       <c r="D389" s="9" t="n">
-        <v>983790</v>
-      </c>
-      <c r="E389" s="6" t="inlineStr"/>
+        <v>6620000</v>
+      </c>
+      <c r="E389" s="8" t="n">
+        <v>0.7259</v>
+      </c>
       <c r="F389" s="7" t="n">
-        <v>46.59</v>
+        <v>51.43</v>
       </c>
       <c r="G389" s="7" t="n">
-        <v>2.92</v>
+        <v>15.76</v>
       </c>
       <c r="H389" s="7" t="n">
-        <v>2.48</v>
+        <v>2.44</v>
       </c>
       <c r="I389" s="8" t="n">
-        <v>1.1538</v>
+        <v>0.1794</v>
       </c>
       <c r="J389" s="8" t="n">
-        <v>1.7569</v>
+        <v>-0.9131999999999999</v>
       </c>
       <c r="K389" s="6" t="inlineStr">
         <is>
@@ -17438,7 +17436,7 @@
       </c>
       <c r="L389" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HOLDING VE YATIRIM, BIST MALİ, BIST İSTANBUL, BIST ANA</t>
+          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST 50, BIST TİCARET, BIST HİZMETLER, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST TEMETTU 25, BIST TEMETTU, BIST KATILIM 50, BIST SÜRDÜRÜLEBİLİRLİK, BIST KATILIM 30, BIST 50-30, BIST KATILIM TEMETTU, BIST SÜRDÜRÜLEBİLİRLİK 25, BIST KATILIM SÜRDÜRÜLEBİLİRLİİK, BIST KATILIM 30 EŞİT AĞIRLIKLI GETİRİ, BIST 50-30 AGIRLIK SINIRLAMALI 25, BIST 50-30 AĞIRLIK SINIRLAMALI 10</t>
         </is>
       </c>
       <c r="M389" s="6" t="inlineStr"/>
@@ -17446,44 +17444,42 @@
     <row r="390">
       <c r="A390" s="2" t="inlineStr">
         <is>
-          <t>MPARK</t>
+          <t>DUNYH</t>
         </is>
       </c>
       <c r="B390" s="3" t="n">
-        <v>455</v>
+        <v>106</v>
       </c>
       <c r="C390" s="4" t="n">
-        <v>0.0271</v>
+        <v>-0.0594</v>
       </c>
       <c r="D390" s="5" t="n">
-        <v>582690</v>
-      </c>
-      <c r="E390" s="4" t="n">
-        <v>0.2922</v>
-      </c>
+        <v>983790</v>
+      </c>
+      <c r="E390" s="2" t="inlineStr"/>
       <c r="F390" s="3" t="n">
-        <v>62</v>
+        <v>46.59</v>
       </c>
       <c r="G390" s="3" t="n">
-        <v>16.41</v>
+        <v>2.92</v>
       </c>
       <c r="H390" s="3" t="n">
-        <v>2.5</v>
+        <v>2.48</v>
       </c>
       <c r="I390" s="4" t="n">
-        <v>0.1843</v>
+        <v>1.1538</v>
       </c>
       <c r="J390" s="4" t="n">
-        <v>-0.09699999999999999</v>
+        <v>1.7569</v>
       </c>
       <c r="K390" s="2" t="inlineStr">
         <is>
-          <t>Sağlık hizmetleri</t>
+          <t>Dayanıklı olmayan tüketici ürünleri</t>
         </is>
       </c>
       <c r="L390" s="2" t="inlineStr">
         <is>
-          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST HİZMETLER, BIST İSTANBUL, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50, BIST SÜRDÜRÜLEBİLİRLİK, BIST KATILIM 30, BIST KATILIM SÜRDÜRÜLEBİLİRLİİK, BIST KATILIM 30 EŞİT AĞIRLIKLI GETİRİ, STOXX Emerging Markets 1500</t>
+          <t>BIST TUM-100, BIST TÜM, BIST HOLDING VE YATIRIM, BIST MALİ, BIST İSTANBUL, BIST ANA</t>
         </is>
       </c>
       <c r="M390" s="2" t="inlineStr"/>
@@ -17491,44 +17487,44 @@
     <row r="391">
       <c r="A391" s="6" t="inlineStr">
         <is>
-          <t>FONET</t>
+          <t>MPARK</t>
         </is>
       </c>
       <c r="B391" s="7" t="n">
-        <v>4.54</v>
+        <v>455</v>
       </c>
       <c r="C391" s="8" t="n">
-        <v>-0.0066</v>
+        <v>0.0271</v>
       </c>
       <c r="D391" s="9" t="n">
-        <v>54110000</v>
+        <v>582690</v>
       </c>
       <c r="E391" s="8" t="n">
-        <v>0.6164999999999999</v>
+        <v>0.2922</v>
       </c>
       <c r="F391" s="7" t="n">
-        <v>47.26</v>
+        <v>62</v>
       </c>
       <c r="G391" s="7" t="n">
-        <v>19.3</v>
+        <v>16.41</v>
       </c>
       <c r="H391" s="7" t="n">
-        <v>2.51</v>
+        <v>2.5</v>
       </c>
       <c r="I391" s="8" t="n">
-        <v>0.1565</v>
+        <v>0.1843</v>
       </c>
       <c r="J391" s="8" t="n">
-        <v>0.7060999999999999</v>
+        <v>-0.09699999999999999</v>
       </c>
       <c r="K391" s="6" t="inlineStr">
         <is>
-          <t>Teknoloji hizmetleri</t>
+          <t>Sağlık hizmetleri</t>
         </is>
       </c>
       <c r="L391" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST KATILIM 100, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST ANKARA</t>
+          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST HİZMETLER, BIST İSTANBUL, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50, BIST SÜRDÜRÜLEBİLİRLİK, BIST KATILIM 30, BIST KATILIM SÜRDÜRÜLEBİLİRLİİK, BIST KATILIM 30 EŞİT AĞIRLIKLI GETİRİ, STOXX Emerging Markets 1500</t>
         </is>
       </c>
       <c r="M391" s="6" t="inlineStr"/>
@@ -17536,42 +17532,44 @@
     <row r="392">
       <c r="A392" s="2" t="inlineStr">
         <is>
-          <t>CUSAN</t>
+          <t>FONET</t>
         </is>
       </c>
       <c r="B392" s="3" t="n">
-        <v>26</v>
+        <v>4.54</v>
       </c>
       <c r="C392" s="4" t="n">
-        <v>0.0062</v>
+        <v>-0.0066</v>
       </c>
       <c r="D392" s="5" t="n">
-        <v>1390000</v>
+        <v>54110000</v>
       </c>
       <c r="E392" s="4" t="n">
-        <v>0.2596</v>
+        <v>0.6164999999999999</v>
       </c>
       <c r="F392" s="3" t="n">
-        <v>57.42</v>
-      </c>
-      <c r="G392" s="2" t="inlineStr"/>
+        <v>47.26</v>
+      </c>
+      <c r="G392" s="3" t="n">
+        <v>19.3</v>
+      </c>
       <c r="H392" s="3" t="n">
         <v>2.51</v>
       </c>
       <c r="I392" s="4" t="n">
-        <v>-0.6525</v>
+        <v>0.1565</v>
       </c>
       <c r="J392" s="4" t="n">
-        <v>-2.2369</v>
+        <v>0.7060999999999999</v>
       </c>
       <c r="K392" s="2" t="inlineStr">
         <is>
-          <t>Enerji-dışı mineraller</t>
+          <t>Teknoloji hizmetleri</t>
         </is>
       </c>
       <c r="L392" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST METAL ANA, BIST İSTANBUL, BIST ANA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST KATILIM 100, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST ANKARA</t>
         </is>
       </c>
       <c r="M392" s="2" t="inlineStr"/>
@@ -17579,40 +17577,42 @@
     <row r="393">
       <c r="A393" s="6" t="inlineStr">
         <is>
-          <t>SEKUR</t>
+          <t>CUSAN</t>
         </is>
       </c>
       <c r="B393" s="7" t="n">
-        <v>8.050000000000001</v>
+        <v>26</v>
       </c>
       <c r="C393" s="8" t="n">
-        <v>-0.029</v>
+        <v>0.0062</v>
       </c>
       <c r="D393" s="9" t="n">
-        <v>3930000</v>
+        <v>1390000</v>
       </c>
       <c r="E393" s="8" t="n">
-        <v>0.2139</v>
+        <v>0.2596</v>
       </c>
       <c r="F393" s="7" t="n">
-        <v>70.52</v>
+        <v>57.42</v>
       </c>
       <c r="G393" s="6" t="inlineStr"/>
       <c r="H393" s="7" t="n">
-        <v>2.52</v>
+        <v>2.51</v>
       </c>
       <c r="I393" s="8" t="n">
-        <v>-0.0267</v>
-      </c>
-      <c r="J393" s="6" t="inlineStr"/>
+        <v>-0.6525</v>
+      </c>
+      <c r="J393" s="8" t="n">
+        <v>-2.2369</v>
+      </c>
       <c r="K393" s="6" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
+          <t>Enerji-dışı mineraller</t>
         </is>
       </c>
       <c r="L393" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST KATILIM TÜM</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST METAL ANA, BIST İSTANBUL, BIST ANA</t>
         </is>
       </c>
       <c r="M393" s="6" t="inlineStr"/>
@@ -17620,42 +17620,40 @@
     <row r="394">
       <c r="A394" s="2" t="inlineStr">
         <is>
-          <t>BJKAS</t>
+          <t>SEKUR</t>
         </is>
       </c>
       <c r="B394" s="3" t="n">
-        <v>1.48</v>
+        <v>8.050000000000001</v>
       </c>
       <c r="C394" s="4" t="n">
-        <v>-0.0199</v>
+        <v>-0.029</v>
       </c>
       <c r="D394" s="5" t="n">
-        <v>31640000</v>
+        <v>3930000</v>
       </c>
       <c r="E394" s="4" t="n">
-        <v>0.2988</v>
+        <v>0.2139</v>
       </c>
       <c r="F394" s="3" t="n">
-        <v>47.33</v>
+        <v>70.52</v>
       </c>
       <c r="G394" s="2" t="inlineStr"/>
       <c r="H394" s="3" t="n">
-        <v>2.53</v>
+        <v>2.52</v>
       </c>
       <c r="I394" s="4" t="n">
-        <v>-33.4785</v>
-      </c>
-      <c r="J394" s="4" t="n">
-        <v>-14.3112</v>
-      </c>
+        <v>-0.0267</v>
+      </c>
+      <c r="J394" s="2" t="inlineStr"/>
       <c r="K394" s="2" t="inlineStr">
         <is>
-          <t>Tüketici hizmetleri</t>
+          <t>İşlenebilen endüstriler</t>
         </is>
       </c>
       <c r="L394" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST SPOR, BIST HİZMETLER, BIST İSTANBUL, BIST YILDIZ</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST KATILIM TÜM</t>
         </is>
       </c>
       <c r="M394" s="2" t="inlineStr"/>
@@ -25699,34 +25697,30 @@
     <row r="581">
       <c r="A581" s="6" t="inlineStr">
         <is>
-          <t>BESTE</t>
+          <t>AAGYO</t>
         </is>
       </c>
       <c r="B581" s="7" t="n">
-        <v>23.4</v>
+        <v>23.24</v>
       </c>
       <c r="C581" s="8" t="n">
-        <v>-0.0059</v>
-      </c>
-      <c r="D581" s="9" t="n">
-        <v>16520000</v>
-      </c>
+        <v>-0.08929999999999999</v>
+      </c>
+      <c r="D581" s="6" t="inlineStr"/>
       <c r="E581" s="6" t="inlineStr"/>
-      <c r="F581" s="7" t="n">
-        <v>53.37</v>
-      </c>
+      <c r="F581" s="6" t="inlineStr"/>
       <c r="G581" s="6" t="inlineStr"/>
       <c r="H581" s="6" t="inlineStr"/>
       <c r="I581" s="6" t="inlineStr"/>
       <c r="J581" s="6" t="inlineStr"/>
       <c r="K581" s="6" t="inlineStr">
         <is>
-          <t>Elektrik, Su, Gaz Hizmetleri</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L581" s="6" t="inlineStr">
         <is>
-          <t>BIST ELEKTRIK, BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST YILDIZ</t>
         </is>
       </c>
       <c r="M581" s="6" t="inlineStr"/>
@@ -25734,23 +25728,23 @@
     <row r="582">
       <c r="A582" s="2" t="inlineStr">
         <is>
-          <t>ICUGS</t>
+          <t>AKGRT</t>
         </is>
       </c>
       <c r="B582" s="3" t="n">
-        <v>3.91</v>
+        <v>7.43</v>
       </c>
       <c r="C582" s="4" t="n">
-        <v>0.0654</v>
+        <v>-0.0107</v>
       </c>
       <c r="D582" s="5" t="n">
-        <v>69940000</v>
+        <v>12600000</v>
       </c>
       <c r="E582" s="4" t="n">
-        <v>0.8667</v>
+        <v>0.28</v>
       </c>
       <c r="F582" s="3" t="n">
-        <v>68.12</v>
+        <v>48.48</v>
       </c>
       <c r="G582" s="2" t="inlineStr"/>
       <c r="H582" s="2" t="inlineStr"/>
@@ -25763,7 +25757,7 @@
       </c>
       <c r="L582" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HOLDING VE YATIRIM, BIST MALİ, BIST ANA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST SİGORTA, BIST MALİ, BIST YILDIZ, BIST SÜRDÜRÜLEBİLİRLİK</t>
         </is>
       </c>
       <c r="M582" s="2" t="inlineStr"/>
@@ -25771,29 +25765,35 @@
     <row r="583">
       <c r="A583" s="6" t="inlineStr">
         <is>
-          <t>DMLKT</t>
+          <t>MMCAS</t>
         </is>
       </c>
       <c r="B583" s="7" t="n">
-        <v>6.28</v>
+        <v>79.90000000000001</v>
       </c>
       <c r="C583" s="8" t="n">
-        <v>-0.0048</v>
+        <v>0.0296</v>
       </c>
       <c r="D583" s="9" t="n">
-        <v>14350000</v>
-      </c>
-      <c r="E583" s="6" t="inlineStr"/>
+        <v>32000</v>
+      </c>
+      <c r="E583" s="8" t="n">
+        <v>0.58</v>
+      </c>
       <c r="F583" s="7" t="n">
-        <v>83.08</v>
+        <v>36.74</v>
       </c>
       <c r="G583" s="6" t="inlineStr"/>
       <c r="H583" s="6" t="inlineStr"/>
-      <c r="I583" s="6" t="inlineStr"/>
-      <c r="J583" s="6" t="inlineStr"/>
+      <c r="I583" s="8" t="n">
+        <v>-9.409700000000001</v>
+      </c>
+      <c r="J583" s="8" t="n">
+        <v>-4.155</v>
+      </c>
       <c r="K583" s="6" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Taşımacılık</t>
         </is>
       </c>
       <c r="L583" s="6" t="inlineStr"/>
@@ -25802,42 +25802,40 @@
     <row r="584">
       <c r="A584" s="2" t="inlineStr">
         <is>
-          <t>BERA</t>
+          <t>BORLS</t>
         </is>
       </c>
       <c r="B584" s="3" t="n">
-        <v>17.21</v>
+        <v>4.38</v>
       </c>
       <c r="C584" s="4" t="n">
-        <v>-0.0205</v>
+        <v>0.0977</v>
       </c>
       <c r="D584" s="5" t="n">
-        <v>12540000</v>
+        <v>39060000</v>
       </c>
       <c r="E584" s="4" t="n">
-        <v>0.9246</v>
+        <v>0.1672</v>
       </c>
       <c r="F584" s="3" t="n">
-        <v>46.95</v>
-      </c>
-      <c r="G584" s="3" t="n">
-        <v>162.67</v>
-      </c>
+        <v>81.56</v>
+      </c>
+      <c r="G584" s="2" t="inlineStr"/>
       <c r="H584" s="2" t="inlineStr"/>
       <c r="I584" s="4" t="n">
-        <v>0.0028</v>
+        <v>-5.3262</v>
       </c>
       <c r="J584" s="4" t="n">
-        <v>-10.3171</v>
+        <v>-4.2562</v>
       </c>
       <c r="K584" s="2" t="inlineStr">
         <is>
-          <t>Üretici imalatı</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L584" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HOLDING VE YATIRIM, BIST MALİ, BIST KATILIM 100, BIST KATILIM TÜM, BIST YILDIZ, BIST KATILIM 50, BIST KONYA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST HİZMETLER, BIST İSTANBUL, BIST YILDIZ</t>
         </is>
       </c>
       <c r="M584" s="2" t="inlineStr"/>
@@ -25845,34 +25843,42 @@
     <row r="585">
       <c r="A585" s="6" t="inlineStr">
         <is>
-          <t>LXGYO</t>
+          <t>BERA</t>
         </is>
       </c>
       <c r="B585" s="7" t="n">
-        <v>15.85</v>
+        <v>17.21</v>
       </c>
       <c r="C585" s="8" t="n">
-        <v>-0.0682</v>
+        <v>-0.0205</v>
       </c>
       <c r="D585" s="9" t="n">
-        <v>120100000</v>
-      </c>
-      <c r="E585" s="6" t="inlineStr"/>
+        <v>12540000</v>
+      </c>
+      <c r="E585" s="8" t="n">
+        <v>0.9246</v>
+      </c>
       <c r="F585" s="7" t="n">
-        <v>51.61</v>
-      </c>
-      <c r="G585" s="6" t="inlineStr"/>
+        <v>46.95</v>
+      </c>
+      <c r="G585" s="7" t="n">
+        <v>162.67</v>
+      </c>
       <c r="H585" s="6" t="inlineStr"/>
-      <c r="I585" s="6" t="inlineStr"/>
-      <c r="J585" s="6" t="inlineStr"/>
+      <c r="I585" s="8" t="n">
+        <v>0.0028</v>
+      </c>
+      <c r="J585" s="8" t="n">
+        <v>-10.3171</v>
+      </c>
       <c r="K585" s="6" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Üretici imalatı</t>
         </is>
       </c>
       <c r="L585" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST ANA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST HOLDING VE YATIRIM, BIST MALİ, BIST KATILIM 100, BIST KATILIM TÜM, BIST YILDIZ, BIST KATILIM 50, BIST KONYA</t>
         </is>
       </c>
       <c r="M585" s="6" t="inlineStr"/>
@@ -25880,67 +25886,69 @@
     <row r="586">
       <c r="A586" s="2" t="inlineStr">
         <is>
-          <t>ALTIN</t>
+          <t>GENKM</t>
         </is>
       </c>
       <c r="B586" s="3" t="n">
-        <v>80.59999999999999</v>
+        <v>13.48</v>
       </c>
       <c r="C586" s="4" t="n">
-        <v>-0.0154</v>
+        <v>-0.0288</v>
       </c>
       <c r="D586" s="5" t="n">
-        <v>12490000</v>
+        <v>60540000</v>
       </c>
       <c r="E586" s="2" t="inlineStr"/>
       <c r="F586" s="3" t="n">
-        <v>39.07</v>
+        <v>52.54</v>
       </c>
       <c r="G586" s="2" t="inlineStr"/>
       <c r="H586" s="2" t="inlineStr"/>
       <c r="I586" s="2" t="inlineStr"/>
       <c r="J586" s="2" t="inlineStr"/>
-      <c r="K586" s="2" t="inlineStr"/>
-      <c r="L586" s="2" t="inlineStr"/>
+      <c r="K586" s="2" t="inlineStr">
+        <is>
+          <t>İşlenebilen endüstriler</t>
+        </is>
+      </c>
+      <c r="L586" s="2" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST KOCAELI</t>
+        </is>
+      </c>
       <c r="M586" s="2" t="inlineStr"/>
     </row>
     <row r="587">
       <c r="A587" s="6" t="inlineStr">
         <is>
-          <t>CRFSA</t>
+          <t>SMRVA</t>
         </is>
       </c>
       <c r="B587" s="7" t="n">
-        <v>166.6</v>
+        <v>82.5</v>
       </c>
       <c r="C587" s="8" t="n">
-        <v>0.08039999999999999</v>
+        <v>0.1</v>
       </c>
       <c r="D587" s="9" t="n">
-        <v>1310000</v>
-      </c>
-      <c r="E587" s="8" t="n">
-        <v>0.1071</v>
-      </c>
+        <v>6190000</v>
+      </c>
+      <c r="E587" s="6" t="inlineStr"/>
       <c r="F587" s="7" t="n">
-        <v>77.11</v>
+        <v>73.01000000000001</v>
       </c>
       <c r="G587" s="6" t="inlineStr"/>
       <c r="H587" s="6" t="inlineStr"/>
-      <c r="I587" s="8" t="n">
-        <v>-3.6635</v>
-      </c>
-      <c r="J587" s="8" t="n">
-        <v>-0.4897</v>
-      </c>
+      <c r="I587" s="6" t="inlineStr"/>
+      <c r="J587" s="6" t="inlineStr"/>
       <c r="K587" s="6" t="inlineStr">
         <is>
-          <t>Perakende satış</t>
+          <t>Ticari hizmetler</t>
         </is>
       </c>
       <c r="L587" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST ANA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST MALİ, BIST ANA, BIST TEMETTU</t>
         </is>
       </c>
       <c r="M587" s="6" t="inlineStr"/>
@@ -25948,56 +25956,48 @@
     <row r="588">
       <c r="A588" s="2" t="inlineStr">
         <is>
-          <t>CGCAM</t>
+          <t>ENPRA</t>
         </is>
       </c>
       <c r="B588" s="3" t="n">
-        <v>36.48</v>
+        <v>112.4</v>
       </c>
       <c r="C588" s="4" t="n">
-        <v>-0.0375</v>
-      </c>
-      <c r="D588" s="5" t="n">
-        <v>6760000</v>
-      </c>
+        <v>-0.09939999999999999</v>
+      </c>
+      <c r="D588" s="2" t="inlineStr"/>
       <c r="E588" s="2" t="inlineStr"/>
-      <c r="F588" s="3" t="n">
-        <v>50.48</v>
-      </c>
+      <c r="F588" s="2" t="inlineStr"/>
       <c r="G588" s="2" t="inlineStr"/>
       <c r="H588" s="2" t="inlineStr"/>
       <c r="I588" s="2" t="inlineStr"/>
       <c r="J588" s="2" t="inlineStr"/>
       <c r="K588" s="2" t="inlineStr">
         <is>
-          <t>Dayanıklı tüketim malları</t>
-        </is>
-      </c>
-      <c r="L588" s="2" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST TAŞ TOPRAK, BIST HALKA ARZ, BIST ANA, BIST MANİSA</t>
-        </is>
-      </c>
+          <t>Finans</t>
+        </is>
+      </c>
+      <c r="L588" s="2" t="inlineStr"/>
       <c r="M588" s="2" t="inlineStr"/>
     </row>
     <row r="589">
       <c r="A589" s="6" t="inlineStr">
         <is>
-          <t>MARMR</t>
+          <t>EMPAE</t>
         </is>
       </c>
       <c r="B589" s="7" t="n">
-        <v>2.85</v>
+        <v>40.02</v>
       </c>
       <c r="C589" s="8" t="n">
-        <v>-0.0404</v>
+        <v>-0.0471</v>
       </c>
       <c r="D589" s="9" t="n">
-        <v>328740000</v>
+        <v>17300000</v>
       </c>
       <c r="E589" s="6" t="inlineStr"/>
       <c r="F589" s="7" t="n">
-        <v>58.27</v>
+        <v>53.04</v>
       </c>
       <c r="G589" s="6" t="inlineStr"/>
       <c r="H589" s="6" t="inlineStr"/>
@@ -26005,12 +26005,12 @@
       <c r="J589" s="6" t="inlineStr"/>
       <c r="K589" s="6" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Elektronik teknoloji</t>
         </is>
       </c>
       <c r="L589" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST ANA, BIST KOCAELI</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI</t>
         </is>
       </c>
       <c r="M589" s="6" t="inlineStr"/>
@@ -26018,34 +26018,38 @@
     <row r="590">
       <c r="A590" s="2" t="inlineStr">
         <is>
-          <t>SMRVA</t>
+          <t>EFOR</t>
         </is>
       </c>
       <c r="B590" s="3" t="n">
-        <v>82.5</v>
+        <v>5.57</v>
       </c>
       <c r="C590" s="4" t="n">
-        <v>0.1</v>
+        <v>0.0431</v>
       </c>
       <c r="D590" s="5" t="n">
-        <v>6190000</v>
-      </c>
-      <c r="E590" s="2" t="inlineStr"/>
+        <v>185340000</v>
+      </c>
+      <c r="E590" s="4" t="n">
+        <v>0.2478</v>
+      </c>
       <c r="F590" s="3" t="n">
-        <v>73.01000000000001</v>
+        <v>15.58</v>
       </c>
       <c r="G590" s="2" t="inlineStr"/>
       <c r="H590" s="2" t="inlineStr"/>
-      <c r="I590" s="2" t="inlineStr"/>
+      <c r="I590" s="4" t="n">
+        <v>-0.0005999999999999999</v>
+      </c>
       <c r="J590" s="2" t="inlineStr"/>
       <c r="K590" s="2" t="inlineStr">
         <is>
-          <t>Ticari hizmetler</t>
+          <t>Dayanıklı olmayan tüketici ürünleri</t>
         </is>
       </c>
       <c r="L590" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST MALİ, BIST ANA, BIST TEMETTU</t>
+          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST GIDA ICECEK, BIST SINAI, BIST TÜM, BIST HALKA ARZ, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50</t>
         </is>
       </c>
       <c r="M590" s="2" t="inlineStr"/>
@@ -26053,38 +26057,34 @@
     <row r="591">
       <c r="A591" s="6" t="inlineStr">
         <is>
-          <t>EFOR</t>
+          <t>GLRMK</t>
         </is>
       </c>
       <c r="B591" s="7" t="n">
-        <v>5.57</v>
+        <v>232</v>
       </c>
       <c r="C591" s="8" t="n">
-        <v>0.0431</v>
+        <v>-0.0353</v>
       </c>
       <c r="D591" s="9" t="n">
-        <v>185340000</v>
-      </c>
-      <c r="E591" s="8" t="n">
-        <v>0.2478</v>
-      </c>
+        <v>14610000</v>
+      </c>
+      <c r="E591" s="6" t="inlineStr"/>
       <c r="F591" s="7" t="n">
-        <v>15.58</v>
+        <v>73.84</v>
       </c>
       <c r="G591" s="6" t="inlineStr"/>
       <c r="H591" s="6" t="inlineStr"/>
-      <c r="I591" s="8" t="n">
-        <v>-0.0005999999999999999</v>
-      </c>
+      <c r="I591" s="6" t="inlineStr"/>
       <c r="J591" s="6" t="inlineStr"/>
       <c r="K591" s="6" t="inlineStr">
         <is>
-          <t>Dayanıklı olmayan tüketici ürünleri</t>
+          <t>Endüstriyel hizmetler</t>
         </is>
       </c>
       <c r="L591" s="6" t="inlineStr">
         <is>
-          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST GIDA ICECEK, BIST SINAI, BIST TÜM, BIST HALKA ARZ, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50</t>
+          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50, BIST KATILIM 30, BIST ANKARA, BIST KATILIM 30 EŞİT AĞIRLIKLI GETİRİ</t>
         </is>
       </c>
       <c r="M591" s="6" t="inlineStr"/>
@@ -26092,40 +26092,36 @@
     <row r="592">
       <c r="A592" s="2" t="inlineStr">
         <is>
-          <t>BORLS</t>
+          <t>UCAYM</t>
         </is>
       </c>
       <c r="B592" s="3" t="n">
-        <v>4.38</v>
+        <v>29.72</v>
       </c>
       <c r="C592" s="4" t="n">
-        <v>0.0977</v>
+        <v>0.0599</v>
       </c>
       <c r="D592" s="5" t="n">
-        <v>39060000</v>
+        <v>11110000</v>
       </c>
       <c r="E592" s="4" t="n">
-        <v>0.1672</v>
+        <v>0.2667</v>
       </c>
       <c r="F592" s="3" t="n">
-        <v>81.56</v>
+        <v>61.87</v>
       </c>
       <c r="G592" s="2" t="inlineStr"/>
       <c r="H592" s="2" t="inlineStr"/>
-      <c r="I592" s="4" t="n">
-        <v>-5.3262</v>
-      </c>
-      <c r="J592" s="4" t="n">
-        <v>-4.2562</v>
-      </c>
+      <c r="I592" s="2" t="inlineStr"/>
+      <c r="J592" s="2" t="inlineStr"/>
       <c r="K592" s="2" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Endüstriyel hizmetler</t>
         </is>
       </c>
       <c r="L592" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HİZMETLER, BIST İSTANBUL, BIST YILDIZ</t>
+          <t>BIST TUM-100, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
         </is>
       </c>
       <c r="M592" s="2" t="inlineStr"/>
@@ -26133,38 +26129,34 @@
     <row r="593">
       <c r="A593" s="6" t="inlineStr">
         <is>
-          <t>NETAS</t>
+          <t>FRMPL</t>
         </is>
       </c>
       <c r="B593" s="7" t="n">
-        <v>61</v>
+        <v>32.96</v>
       </c>
       <c r="C593" s="8" t="n">
-        <v>-0.0224</v>
+        <v>-0.009000000000000001</v>
       </c>
       <c r="D593" s="9" t="n">
-        <v>1050000</v>
-      </c>
-      <c r="E593" s="8" t="n">
-        <v>0.3695000000000001</v>
-      </c>
+        <v>5490000</v>
+      </c>
+      <c r="E593" s="6" t="inlineStr"/>
       <c r="F593" s="7" t="n">
-        <v>54.08</v>
+        <v>52.75</v>
       </c>
       <c r="G593" s="6" t="inlineStr"/>
       <c r="H593" s="6" t="inlineStr"/>
       <c r="I593" s="6" t="inlineStr"/>
-      <c r="J593" s="8" t="n">
-        <v>0.4139</v>
-      </c>
+      <c r="J593" s="6" t="inlineStr"/>
       <c r="K593" s="6" t="inlineStr">
         <is>
-          <t>Teknoloji hizmetleri</t>
+          <t>Üretici imalatı</t>
         </is>
       </c>
       <c r="L593" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST İSTANBUL, BIST KATILIM 100, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KURUMSAL YÖNETİM</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST TEKİRDAĞ</t>
         </is>
       </c>
       <c r="M593" s="6" t="inlineStr"/>
@@ -26172,34 +26164,38 @@
     <row r="594">
       <c r="A594" s="2" t="inlineStr">
         <is>
-          <t>FRMPL</t>
+          <t>NETAS</t>
         </is>
       </c>
       <c r="B594" s="3" t="n">
-        <v>32.96</v>
+        <v>61</v>
       </c>
       <c r="C594" s="4" t="n">
-        <v>-0.009000000000000001</v>
+        <v>-0.0224</v>
       </c>
       <c r="D594" s="5" t="n">
-        <v>5490000</v>
-      </c>
-      <c r="E594" s="2" t="inlineStr"/>
+        <v>1050000</v>
+      </c>
+      <c r="E594" s="4" t="n">
+        <v>0.3695000000000001</v>
+      </c>
       <c r="F594" s="3" t="n">
-        <v>52.75</v>
+        <v>54.08</v>
       </c>
       <c r="G594" s="2" t="inlineStr"/>
       <c r="H594" s="2" t="inlineStr"/>
       <c r="I594" s="2" t="inlineStr"/>
-      <c r="J594" s="2" t="inlineStr"/>
+      <c r="J594" s="4" t="n">
+        <v>0.4139</v>
+      </c>
       <c r="K594" s="2" t="inlineStr">
         <is>
-          <t>Üretici imalatı</t>
+          <t>Teknoloji hizmetleri</t>
         </is>
       </c>
       <c r="L594" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST TEKİRDAĞ</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST İSTANBUL, BIST KATILIM 100, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KURUMSAL YÖNETİM</t>
         </is>
       </c>
       <c r="M594" s="2" t="inlineStr"/>
@@ -26207,21 +26203,23 @@
     <row r="595">
       <c r="A595" s="6" t="inlineStr">
         <is>
-          <t>SVGYO</t>
+          <t>INTEK</t>
         </is>
       </c>
       <c r="B595" s="7" t="n">
-        <v>16.35</v>
+        <v>254</v>
       </c>
       <c r="C595" s="8" t="n">
-        <v>-0.09970000000000001</v>
+        <v>0.0292</v>
       </c>
       <c r="D595" s="9" t="n">
-        <v>87640000</v>
-      </c>
-      <c r="E595" s="6" t="inlineStr"/>
+        <v>8560</v>
+      </c>
+      <c r="E595" s="8" t="n">
+        <v>0.2578</v>
+      </c>
       <c r="F595" s="7" t="n">
-        <v>76.05</v>
+        <v>49.66</v>
       </c>
       <c r="G595" s="6" t="inlineStr"/>
       <c r="H595" s="6" t="inlineStr"/>
@@ -26229,90 +26227,78 @@
       <c r="J595" s="6" t="inlineStr"/>
       <c r="K595" s="6" t="inlineStr">
         <is>
-          <t>Finans</t>
-        </is>
-      </c>
-      <c r="L595" s="6" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST ANA</t>
-        </is>
-      </c>
+          <t>İşlenebilen endüstriler</t>
+        </is>
+      </c>
+      <c r="L595" s="6" t="inlineStr"/>
       <c r="M595" s="6" t="inlineStr"/>
     </row>
     <row r="596">
       <c r="A596" s="2" t="inlineStr">
         <is>
-          <t>MMCAS</t>
+          <t>CGCAM</t>
         </is>
       </c>
       <c r="B596" s="3" t="n">
-        <v>79.90000000000001</v>
+        <v>36.48</v>
       </c>
       <c r="C596" s="4" t="n">
-        <v>0.0296</v>
+        <v>-0.0375</v>
       </c>
       <c r="D596" s="5" t="n">
-        <v>32000</v>
-      </c>
-      <c r="E596" s="4" t="n">
-        <v>0.58</v>
-      </c>
+        <v>6760000</v>
+      </c>
+      <c r="E596" s="2" t="inlineStr"/>
       <c r="F596" s="3" t="n">
-        <v>36.74</v>
+        <v>50.48</v>
       </c>
       <c r="G596" s="2" t="inlineStr"/>
       <c r="H596" s="2" t="inlineStr"/>
-      <c r="I596" s="4" t="n">
-        <v>-9.409700000000001</v>
-      </c>
-      <c r="J596" s="4" t="n">
-        <v>-4.155</v>
-      </c>
+      <c r="I596" s="2" t="inlineStr"/>
+      <c r="J596" s="2" t="inlineStr"/>
       <c r="K596" s="2" t="inlineStr">
         <is>
-          <t>Taşımacılık</t>
-        </is>
-      </c>
-      <c r="L596" s="2" t="inlineStr"/>
+          <t>Dayanıklı tüketim malları</t>
+        </is>
+      </c>
+      <c r="L596" s="2" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST TAŞ TOPRAK, BIST HALKA ARZ, BIST ANA, BIST MANİSA</t>
+        </is>
+      </c>
       <c r="M596" s="2" t="inlineStr"/>
     </row>
     <row r="597">
       <c r="A597" s="6" t="inlineStr">
         <is>
-          <t>ARZUM</t>
+          <t>LXGYO</t>
         </is>
       </c>
       <c r="B597" s="7" t="n">
-        <v>3.27</v>
+        <v>15.85</v>
       </c>
       <c r="C597" s="8" t="n">
-        <v>-0.0325</v>
+        <v>-0.0682</v>
       </c>
       <c r="D597" s="9" t="n">
-        <v>73930000</v>
-      </c>
-      <c r="E597" s="8" t="n">
-        <v>0.7119</v>
-      </c>
+        <v>120100000</v>
+      </c>
+      <c r="E597" s="6" t="inlineStr"/>
       <c r="F597" s="7" t="n">
-        <v>62.53</v>
+        <v>51.61</v>
       </c>
       <c r="G597" s="6" t="inlineStr"/>
       <c r="H597" s="6" t="inlineStr"/>
-      <c r="I597" s="8" t="n">
-        <v>-191.6342</v>
-      </c>
-      <c r="J597" s="8" t="n">
-        <v>-0.8093</v>
-      </c>
+      <c r="I597" s="6" t="inlineStr"/>
+      <c r="J597" s="6" t="inlineStr"/>
       <c r="K597" s="6" t="inlineStr">
         <is>
-          <t>Dağıtım servisleri</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L597" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST İSTANBUL, BIST ANA, BIST KURUMSAL YÖNETİM</t>
+          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST ANA</t>
         </is>
       </c>
       <c r="M597" s="6" t="inlineStr"/>
@@ -26320,18 +26306,22 @@
     <row r="598">
       <c r="A598" s="2" t="inlineStr">
         <is>
-          <t>AAGYO</t>
+          <t>SVGYO</t>
         </is>
       </c>
       <c r="B598" s="3" t="n">
-        <v>23.24</v>
+        <v>16.35</v>
       </c>
       <c r="C598" s="4" t="n">
-        <v>-0.08929999999999999</v>
-      </c>
-      <c r="D598" s="2" t="inlineStr"/>
+        <v>-0.09970000000000001</v>
+      </c>
+      <c r="D598" s="5" t="n">
+        <v>87640000</v>
+      </c>
       <c r="E598" s="2" t="inlineStr"/>
-      <c r="F598" s="2" t="inlineStr"/>
+      <c r="F598" s="3" t="n">
+        <v>76.05</v>
+      </c>
       <c r="G598" s="2" t="inlineStr"/>
       <c r="H598" s="2" t="inlineStr"/>
       <c r="I598" s="2" t="inlineStr"/>
@@ -26343,7 +26333,7 @@
       </c>
       <c r="L598" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST YILDIZ</t>
+          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST ANA</t>
         </is>
       </c>
       <c r="M598" s="2" t="inlineStr"/>
@@ -26351,21 +26341,21 @@
     <row r="599">
       <c r="A599" s="6" t="inlineStr">
         <is>
-          <t>EMPAE</t>
+          <t>DMLKT</t>
         </is>
       </c>
       <c r="B599" s="7" t="n">
-        <v>40.02</v>
+        <v>6.28</v>
       </c>
       <c r="C599" s="8" t="n">
-        <v>-0.0471</v>
+        <v>-0.0048</v>
       </c>
       <c r="D599" s="9" t="n">
-        <v>17300000</v>
+        <v>14350000</v>
       </c>
       <c r="E599" s="6" t="inlineStr"/>
       <c r="F599" s="7" t="n">
-        <v>53.04</v>
+        <v>83.08</v>
       </c>
       <c r="G599" s="6" t="inlineStr"/>
       <c r="H599" s="6" t="inlineStr"/>
@@ -26373,98 +26363,100 @@
       <c r="J599" s="6" t="inlineStr"/>
       <c r="K599" s="6" t="inlineStr">
         <is>
-          <t>Elektronik teknoloji</t>
-        </is>
-      </c>
-      <c r="L599" s="6" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI</t>
-        </is>
-      </c>
+          <t>Finans</t>
+        </is>
+      </c>
+      <c r="L599" s="6" t="inlineStr"/>
       <c r="M599" s="6" t="inlineStr"/>
     </row>
     <row r="600">
       <c r="A600" s="2" t="inlineStr">
         <is>
-          <t>ENPRA</t>
+          <t>CRFSA</t>
         </is>
       </c>
       <c r="B600" s="3" t="n">
-        <v>112.4</v>
+        <v>166.6</v>
       </c>
       <c r="C600" s="4" t="n">
-        <v>-0.09939999999999999</v>
-      </c>
-      <c r="D600" s="2" t="inlineStr"/>
-      <c r="E600" s="2" t="inlineStr"/>
-      <c r="F600" s="2" t="inlineStr"/>
+        <v>0.08039999999999999</v>
+      </c>
+      <c r="D600" s="5" t="n">
+        <v>1310000</v>
+      </c>
+      <c r="E600" s="4" t="n">
+        <v>0.1071</v>
+      </c>
+      <c r="F600" s="3" t="n">
+        <v>77.11</v>
+      </c>
       <c r="G600" s="2" t="inlineStr"/>
       <c r="H600" s="2" t="inlineStr"/>
-      <c r="I600" s="2" t="inlineStr"/>
-      <c r="J600" s="2" t="inlineStr"/>
+      <c r="I600" s="4" t="n">
+        <v>-3.6635</v>
+      </c>
+      <c r="J600" s="4" t="n">
+        <v>-0.4897</v>
+      </c>
       <c r="K600" s="2" t="inlineStr">
         <is>
-          <t>Finans</t>
-        </is>
-      </c>
-      <c r="L600" s="2" t="inlineStr"/>
+          <t>Perakende satış</t>
+        </is>
+      </c>
+      <c r="L600" s="2" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST ANA</t>
+        </is>
+      </c>
       <c r="M600" s="2" t="inlineStr"/>
     </row>
     <row r="601">
       <c r="A601" s="6" t="inlineStr">
         <is>
-          <t>MCARD</t>
+          <t>ALTIN</t>
         </is>
       </c>
       <c r="B601" s="7" t="n">
-        <v>197</v>
+        <v>80.59999999999999</v>
       </c>
       <c r="C601" s="8" t="n">
-        <v>0.0336</v>
+        <v>-0.0154</v>
       </c>
       <c r="D601" s="9" t="n">
-        <v>14110000</v>
+        <v>12490000</v>
       </c>
       <c r="E601" s="6" t="inlineStr"/>
       <c r="F601" s="7" t="n">
-        <v>77.95999999999999</v>
+        <v>39.07</v>
       </c>
       <c r="G601" s="6" t="inlineStr"/>
       <c r="H601" s="6" t="inlineStr"/>
       <c r="I601" s="6" t="inlineStr"/>
       <c r="J601" s="6" t="inlineStr"/>
-      <c r="K601" s="6" t="inlineStr">
-        <is>
-          <t>Ticari hizmetler</t>
-        </is>
-      </c>
-      <c r="L601" s="6" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI</t>
-        </is>
-      </c>
+      <c r="K601" s="6" t="inlineStr"/>
+      <c r="L601" s="6" t="inlineStr"/>
       <c r="M601" s="6" t="inlineStr"/>
     </row>
     <row r="602">
       <c r="A602" s="2" t="inlineStr">
         <is>
-          <t>UCAYM</t>
+          <t>ICUGS</t>
         </is>
       </c>
       <c r="B602" s="3" t="n">
-        <v>29.72</v>
+        <v>3.91</v>
       </c>
       <c r="C602" s="4" t="n">
-        <v>0.0599</v>
+        <v>0.0654</v>
       </c>
       <c r="D602" s="5" t="n">
-        <v>11110000</v>
+        <v>69940000</v>
       </c>
       <c r="E602" s="4" t="n">
-        <v>0.2667</v>
+        <v>0.8667</v>
       </c>
       <c r="F602" s="3" t="n">
-        <v>61.87</v>
+        <v>68.12</v>
       </c>
       <c r="G602" s="2" t="inlineStr"/>
       <c r="H602" s="2" t="inlineStr"/>
@@ -26472,12 +26464,12 @@
       <c r="J602" s="2" t="inlineStr"/>
       <c r="K602" s="2" t="inlineStr">
         <is>
-          <t>Endüstriyel hizmetler</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L602" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST HOLDING VE YATIRIM, BIST MALİ, BIST ANA</t>
         </is>
       </c>
       <c r="M602" s="2" t="inlineStr"/>
@@ -26485,58 +26477,62 @@
     <row r="603">
       <c r="A603" s="6" t="inlineStr">
         <is>
-          <t>BRMEN</t>
+          <t>ARZUM</t>
         </is>
       </c>
       <c r="B603" s="7" t="n">
-        <v>10</v>
+        <v>3.27</v>
       </c>
       <c r="C603" s="8" t="n">
-        <v>-0.0476</v>
+        <v>-0.0325</v>
       </c>
       <c r="D603" s="9" t="n">
-        <v>266560</v>
+        <v>73930000</v>
       </c>
       <c r="E603" s="8" t="n">
-        <v>0.95</v>
+        <v>0.7119</v>
       </c>
       <c r="F603" s="7" t="n">
-        <v>59.22</v>
+        <v>62.53</v>
       </c>
       <c r="G603" s="6" t="inlineStr"/>
       <c r="H603" s="6" t="inlineStr"/>
       <c r="I603" s="8" t="n">
-        <v>-23.6291</v>
+        <v>-191.6342</v>
       </c>
       <c r="J603" s="8" t="n">
-        <v>-0.4678</v>
+        <v>-0.8093</v>
       </c>
       <c r="K603" s="6" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
-        </is>
-      </c>
-      <c r="L603" s="6" t="inlineStr"/>
+          <t>Dağıtım servisleri</t>
+        </is>
+      </c>
+      <c r="L603" s="6" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST İSTANBUL, BIST ANA, BIST KURUMSAL YÖNETİM</t>
+        </is>
+      </c>
       <c r="M603" s="6" t="inlineStr"/>
     </row>
     <row r="604">
       <c r="A604" s="2" t="inlineStr">
         <is>
-          <t>GLRMK</t>
+          <t>MCARD</t>
         </is>
       </c>
       <c r="B604" s="3" t="n">
-        <v>232</v>
+        <v>197</v>
       </c>
       <c r="C604" s="4" t="n">
-        <v>-0.0353</v>
+        <v>0.0336</v>
       </c>
       <c r="D604" s="5" t="n">
-        <v>14610000</v>
+        <v>14110000</v>
       </c>
       <c r="E604" s="2" t="inlineStr"/>
       <c r="F604" s="3" t="n">
-        <v>73.84</v>
+        <v>77.95999999999999</v>
       </c>
       <c r="G604" s="2" t="inlineStr"/>
       <c r="H604" s="2" t="inlineStr"/>
@@ -26544,12 +26540,12 @@
       <c r="J604" s="2" t="inlineStr"/>
       <c r="K604" s="2" t="inlineStr">
         <is>
-          <t>Endüstriyel hizmetler</t>
+          <t>Ticari hizmetler</t>
         </is>
       </c>
       <c r="L604" s="2" t="inlineStr">
         <is>
-          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50, BIST KATILIM 30, BIST ANKARA, BIST KATILIM 30 EŞİT AĞIRLIKLI GETİRİ</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI</t>
         </is>
       </c>
       <c r="M604" s="2" t="inlineStr"/>
@@ -26557,23 +26553,21 @@
     <row r="605">
       <c r="A605" s="6" t="inlineStr">
         <is>
-          <t>INTEK</t>
+          <t>BESTE</t>
         </is>
       </c>
       <c r="B605" s="7" t="n">
-        <v>254</v>
+        <v>23.4</v>
       </c>
       <c r="C605" s="8" t="n">
-        <v>0.0292</v>
+        <v>-0.0059</v>
       </c>
       <c r="D605" s="9" t="n">
-        <v>8560</v>
-      </c>
-      <c r="E605" s="8" t="n">
-        <v>0.2578</v>
-      </c>
+        <v>16520000</v>
+      </c>
+      <c r="E605" s="6" t="inlineStr"/>
       <c r="F605" s="7" t="n">
-        <v>49.66</v>
+        <v>53.37</v>
       </c>
       <c r="G605" s="6" t="inlineStr"/>
       <c r="H605" s="6" t="inlineStr"/>
@@ -26581,67 +26575,71 @@
       <c r="J605" s="6" t="inlineStr"/>
       <c r="K605" s="6" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
-        </is>
-      </c>
-      <c r="L605" s="6" t="inlineStr"/>
+          <t>Elektrik, Su, Gaz Hizmetleri</t>
+        </is>
+      </c>
+      <c r="L605" s="6" t="inlineStr">
+        <is>
+          <t>BIST ELEKTRIK, BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
+        </is>
+      </c>
       <c r="M605" s="6" t="inlineStr"/>
     </row>
     <row r="606">
       <c r="A606" s="2" t="inlineStr">
         <is>
-          <t>AKGRT</t>
+          <t>BRMEN</t>
         </is>
       </c>
       <c r="B606" s="3" t="n">
-        <v>7.43</v>
+        <v>10</v>
       </c>
       <c r="C606" s="4" t="n">
-        <v>-0.0107</v>
+        <v>-0.0476</v>
       </c>
       <c r="D606" s="5" t="n">
-        <v>12600000</v>
+        <v>266560</v>
       </c>
       <c r="E606" s="4" t="n">
-        <v>0.28</v>
+        <v>0.95</v>
       </c>
       <c r="F606" s="3" t="n">
-        <v>48.48</v>
+        <v>59.22</v>
       </c>
       <c r="G606" s="2" t="inlineStr"/>
       <c r="H606" s="2" t="inlineStr"/>
-      <c r="I606" s="2" t="inlineStr"/>
-      <c r="J606" s="2" t="inlineStr"/>
+      <c r="I606" s="4" t="n">
+        <v>-23.6291</v>
+      </c>
+      <c r="J606" s="4" t="n">
+        <v>-0.4678</v>
+      </c>
       <c r="K606" s="2" t="inlineStr">
         <is>
-          <t>Finans</t>
-        </is>
-      </c>
-      <c r="L606" s="2" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST TÜM, BIST SİGORTA, BIST MALİ, BIST YILDIZ, BIST SÜRDÜRÜLEBİLİRLİK</t>
-        </is>
-      </c>
+          <t>İşlenebilen endüstriler</t>
+        </is>
+      </c>
+      <c r="L606" s="2" t="inlineStr"/>
       <c r="M606" s="2" t="inlineStr"/>
     </row>
     <row r="607">
       <c r="A607" s="6" t="inlineStr">
         <is>
-          <t>GENKM</t>
+          <t>MARMR</t>
         </is>
       </c>
       <c r="B607" s="7" t="n">
-        <v>13.48</v>
+        <v>2.85</v>
       </c>
       <c r="C607" s="8" t="n">
-        <v>-0.0288</v>
+        <v>-0.0404</v>
       </c>
       <c r="D607" s="9" t="n">
-        <v>60540000</v>
+        <v>328740000</v>
       </c>
       <c r="E607" s="6" t="inlineStr"/>
       <c r="F607" s="7" t="n">
-        <v>52.54</v>
+        <v>58.27</v>
       </c>
       <c r="G607" s="6" t="inlineStr"/>
       <c r="H607" s="6" t="inlineStr"/>
@@ -26649,12 +26647,12 @@
       <c r="J607" s="6" t="inlineStr"/>
       <c r="K607" s="6" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L607" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST KOCAELI</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST ANA, BIST KOCAELI</t>
         </is>
       </c>
       <c r="M607" s="6" t="inlineStr"/>
@@ -26681,7 +26679,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>13.04.2026 16:30</t>
+          <t>13.04.2026 19:52</t>
         </is>
       </c>
     </row>

</xml_diff>